<commit_message>
Add 24-month pending-catalyst schedule grid
FDA Decisions Pending gains a schedule status column plus a month-per-column grid
running 2026-09 to 2028-08. Each pending clause is mapped to a month span by
schedule_grid.py and shaded by date precision, so a firm PDUFA date reads
differently from a bare-year guess. Clauses whose window predates the grid are
flagged overdue rather than silently dropped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H18zxCm9b8hEQHez8ngxS5
</commit_message>
<xml_diff>
--- a/FDA_Pipeline_US_Listed.xlsx
+++ b/FDA_Pipeline_US_Listed.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$1:$S$339</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Summary'!$A$1:$M$179</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FDA Decisions Pending'!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'FDA Decisions Pending'!$A$1:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Ticker Watchlist'!$A$1:$M$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,23 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <color rgb="001F1F1F"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <color rgb="00404040"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
@@ -52,7 +69,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +79,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009DC3E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -99,7 +131,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -111,11 +143,32 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -39717,7 +39770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:AJ83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -39731,9 +39784,34 @@
     <col width="52" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="4.2" customWidth="1" min="13" max="13"/>
+    <col width="4.2" customWidth="1" min="14" max="14"/>
+    <col width="4.2" customWidth="1" min="15" max="15"/>
+    <col width="4.2" customWidth="1" min="16" max="16"/>
+    <col width="4.2" customWidth="1" min="17" max="17"/>
+    <col width="4.2" customWidth="1" min="18" max="18"/>
+    <col width="4.2" customWidth="1" min="19" max="19"/>
+    <col width="4.2" customWidth="1" min="20" max="20"/>
+    <col width="4.2" customWidth="1" min="21" max="21"/>
+    <col width="4.2" customWidth="1" min="22" max="22"/>
+    <col width="4.2" customWidth="1" min="23" max="23"/>
+    <col width="4.2" customWidth="1" min="24" max="24"/>
+    <col width="4.2" customWidth="1" min="25" max="25"/>
+    <col width="4.2" customWidth="1" min="26" max="26"/>
+    <col width="4.2" customWidth="1" min="27" max="27"/>
+    <col width="4.2" customWidth="1" min="28" max="28"/>
+    <col width="4.2" customWidth="1" min="29" max="29"/>
+    <col width="4.2" customWidth="1" min="30" max="30"/>
+    <col width="4.2" customWidth="1" min="31" max="31"/>
+    <col width="4.2" customWidth="1" min="32" max="32"/>
+    <col width="4.2" customWidth="1" min="33" max="33"/>
+    <col width="4.2" customWidth="1" min="34" max="34"/>
+    <col width="4.2" customWidth="1" min="35" max="35"/>
+    <col width="4.2" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1" ht="62" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>公司 Company</t>
@@ -39787,6 +39865,131 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註 Notes</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>排程狀態 Schedule status</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="V1" s="7" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="W1" s="7" t="inlineStr">
+        <is>
+          <t>2027-07</t>
+        </is>
+      </c>
+      <c r="X1" s="7" t="inlineStr">
+        <is>
+          <t>2027-08</t>
+        </is>
+      </c>
+      <c r="Y1" s="7" t="inlineStr">
+        <is>
+          <t>2027-09</t>
+        </is>
+      </c>
+      <c r="Z1" s="7" t="inlineStr">
+        <is>
+          <t>2027-10</t>
+        </is>
+      </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
+          <t>2027-11</t>
+        </is>
+      </c>
+      <c r="AB1" s="7" t="inlineStr">
+        <is>
+          <t>2027-12</t>
+        </is>
+      </c>
+      <c r="AC1" s="8" t="inlineStr">
+        <is>
+          <t>2028-01</t>
+        </is>
+      </c>
+      <c r="AD1" s="7" t="inlineStr">
+        <is>
+          <t>2028-02</t>
+        </is>
+      </c>
+      <c r="AE1" s="7" t="inlineStr">
+        <is>
+          <t>2028-03</t>
+        </is>
+      </c>
+      <c r="AF1" s="7" t="inlineStr">
+        <is>
+          <t>2028-04</t>
+        </is>
+      </c>
+      <c r="AG1" s="7" t="inlineStr">
+        <is>
+          <t>2028-05</t>
+        </is>
+      </c>
+      <c r="AH1" s="7" t="inlineStr">
+        <is>
+          <t>2028-06</t>
+        </is>
+      </c>
+      <c r="AI1" s="7" t="inlineStr">
+        <is>
+          <t>2028-07</t>
+        </is>
+      </c>
+      <c r="AJ1" s="7" t="inlineStr">
+        <is>
+          <t>2028-08</t>
         </is>
       </c>
     </row>
@@ -39842,6 +40045,39 @@
           <t>First oral non-peptide GLP-1; ACHIEVE/ATTAIN Ph3 positive</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: 遞交</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N2" s="10" t="n"/>
+      <c r="O2" s="10" t="n"/>
+      <c r="P2" s="10" t="n"/>
+      <c r="Q2" s="11" t="n"/>
+      <c r="R2" s="11" t="n"/>
+      <c r="S2" s="11" t="n"/>
+      <c r="T2" s="11" t="n"/>
+      <c r="U2" s="11" t="n"/>
+      <c r="V2" s="11" t="n"/>
+      <c r="W2" s="11" t="n"/>
+      <c r="X2" s="11" t="n"/>
+      <c r="Y2" s="11" t="n"/>
+      <c r="Z2" s="11" t="n"/>
+      <c r="AA2" s="11" t="n"/>
+      <c r="AB2" s="11" t="n"/>
+      <c r="AC2" s="11" t="n"/>
+      <c r="AD2" s="11" t="n"/>
+      <c r="AE2" s="11" t="n"/>
+      <c r="AF2" s="11" t="n"/>
+      <c r="AG2" s="11" t="n"/>
+      <c r="AH2" s="11" t="n"/>
+      <c r="AI2" s="11" t="n"/>
+      <c r="AJ2" s="11" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -39891,6 +40127,35 @@
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="n"/>
+      <c r="O3" s="10" t="n"/>
+      <c r="P3" s="10" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
+      <c r="T3" s="11" t="n"/>
+      <c r="U3" s="11" t="n"/>
+      <c r="V3" s="11" t="n"/>
+      <c r="W3" s="11" t="n"/>
+      <c r="X3" s="11" t="n"/>
+      <c r="Y3" s="11" t="n"/>
+      <c r="Z3" s="11" t="n"/>
+      <c r="AA3" s="11" t="n"/>
+      <c r="AB3" s="11" t="n"/>
+      <c r="AC3" s="11" t="n"/>
+      <c r="AD3" s="11" t="n"/>
+      <c r="AE3" s="11" t="n"/>
+      <c r="AF3" s="11" t="n"/>
+      <c r="AG3" s="11" t="n"/>
+      <c r="AH3" s="11" t="n"/>
+      <c r="AI3" s="11" t="n"/>
+      <c r="AJ3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -39944,6 +40209,35 @@
           <t>Partnered with Arvinas (ARVN)</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M4" s="11" t="n"/>
+      <c r="N4" s="11" t="n"/>
+      <c r="O4" s="11" t="n"/>
+      <c r="P4" s="11" t="n"/>
+      <c r="Q4" s="11" t="n"/>
+      <c r="R4" s="11" t="n"/>
+      <c r="S4" s="11" t="n"/>
+      <c r="T4" s="11" t="n"/>
+      <c r="U4" s="11" t="n"/>
+      <c r="V4" s="11" t="n"/>
+      <c r="W4" s="11" t="n"/>
+      <c r="X4" s="11" t="n"/>
+      <c r="Y4" s="11" t="n"/>
+      <c r="Z4" s="11" t="n"/>
+      <c r="AA4" s="11" t="n"/>
+      <c r="AB4" s="11" t="n"/>
+      <c r="AC4" s="11" t="n"/>
+      <c r="AD4" s="11" t="n"/>
+      <c r="AE4" s="11" t="n"/>
+      <c r="AF4" s="11" t="n"/>
+      <c r="AG4" s="11" t="n"/>
+      <c r="AH4" s="11" t="n"/>
+      <c r="AI4" s="11" t="n"/>
+      <c r="AJ4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -39997,6 +40291,35 @@
           <t>First oral PCSK9</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="n"/>
+      <c r="O5" s="10" t="n"/>
+      <c r="P5" s="10" t="n"/>
+      <c r="Q5" s="11" t="n"/>
+      <c r="R5" s="11" t="n"/>
+      <c r="S5" s="11" t="n"/>
+      <c r="T5" s="11" t="n"/>
+      <c r="U5" s="11" t="n"/>
+      <c r="V5" s="11" t="n"/>
+      <c r="W5" s="11" t="n"/>
+      <c r="X5" s="11" t="n"/>
+      <c r="Y5" s="11" t="n"/>
+      <c r="Z5" s="11" t="n"/>
+      <c r="AA5" s="11" t="n"/>
+      <c r="AB5" s="11" t="n"/>
+      <c r="AC5" s="11" t="n"/>
+      <c r="AD5" s="11" t="n"/>
+      <c r="AE5" s="11" t="n"/>
+      <c r="AF5" s="11" t="n"/>
+      <c r="AG5" s="11" t="n"/>
+      <c r="AH5" s="11" t="n"/>
+      <c r="AI5" s="11" t="n"/>
+      <c r="AJ5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -40046,6 +40369,35 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N6" s="10" t="n"/>
+      <c r="O6" s="10" t="n"/>
+      <c r="P6" s="10" t="n"/>
+      <c r="Q6" s="11" t="n"/>
+      <c r="R6" s="11" t="n"/>
+      <c r="S6" s="11" t="n"/>
+      <c r="T6" s="11" t="n"/>
+      <c r="U6" s="11" t="n"/>
+      <c r="V6" s="11" t="n"/>
+      <c r="W6" s="11" t="n"/>
+      <c r="X6" s="11" t="n"/>
+      <c r="Y6" s="11" t="n"/>
+      <c r="Z6" s="11" t="n"/>
+      <c r="AA6" s="11" t="n"/>
+      <c r="AB6" s="11" t="n"/>
+      <c r="AC6" s="11" t="n"/>
+      <c r="AD6" s="11" t="n"/>
+      <c r="AE6" s="11" t="n"/>
+      <c r="AF6" s="11" t="n"/>
+      <c r="AG6" s="11" t="n"/>
+      <c r="AH6" s="11" t="n"/>
+      <c r="AI6" s="11" t="n"/>
+      <c r="AJ6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -40099,6 +40451,35 @@
           <t>First oral IL-23</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="n"/>
+      <c r="O7" s="10" t="n"/>
+      <c r="P7" s="10" t="n"/>
+      <c r="Q7" s="11" t="n"/>
+      <c r="R7" s="11" t="n"/>
+      <c r="S7" s="11" t="n"/>
+      <c r="T7" s="11" t="n"/>
+      <c r="U7" s="11" t="n"/>
+      <c r="V7" s="11" t="n"/>
+      <c r="W7" s="11" t="n"/>
+      <c r="X7" s="11" t="n"/>
+      <c r="Y7" s="11" t="n"/>
+      <c r="Z7" s="11" t="n"/>
+      <c r="AA7" s="11" t="n"/>
+      <c r="AB7" s="11" t="n"/>
+      <c r="AC7" s="11" t="n"/>
+      <c r="AD7" s="11" t="n"/>
+      <c r="AE7" s="11" t="n"/>
+      <c r="AF7" s="11" t="n"/>
+      <c r="AG7" s="11" t="n"/>
+      <c r="AH7" s="11" t="n"/>
+      <c r="AI7" s="11" t="n"/>
+      <c r="AJ7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -40148,6 +40529,35 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="n"/>
+      <c r="O8" s="13" t="n"/>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="11" t="n"/>
+      <c r="R8" s="11" t="n"/>
+      <c r="S8" s="11" t="n"/>
+      <c r="T8" s="11" t="n"/>
+      <c r="U8" s="11" t="n"/>
+      <c r="V8" s="11" t="n"/>
+      <c r="W8" s="11" t="n"/>
+      <c r="X8" s="11" t="n"/>
+      <c r="Y8" s="11" t="n"/>
+      <c r="Z8" s="11" t="n"/>
+      <c r="AA8" s="11" t="n"/>
+      <c r="AB8" s="11" t="n"/>
+      <c r="AC8" s="11" t="n"/>
+      <c r="AD8" s="11" t="n"/>
+      <c r="AE8" s="11" t="n"/>
+      <c r="AF8" s="11" t="n"/>
+      <c r="AG8" s="11" t="n"/>
+      <c r="AH8" s="11" t="n"/>
+      <c r="AI8" s="11" t="n"/>
+      <c r="AJ8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -40201,6 +40611,35 @@
           <t>From Cerevel acquisition</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="n"/>
+      <c r="O9" s="10" t="n"/>
+      <c r="P9" s="10" t="n"/>
+      <c r="Q9" s="11" t="n"/>
+      <c r="R9" s="11" t="n"/>
+      <c r="S9" s="11" t="n"/>
+      <c r="T9" s="11" t="n"/>
+      <c r="U9" s="11" t="n"/>
+      <c r="V9" s="11" t="n"/>
+      <c r="W9" s="11" t="n"/>
+      <c r="X9" s="11" t="n"/>
+      <c r="Y9" s="11" t="n"/>
+      <c r="Z9" s="11" t="n"/>
+      <c r="AA9" s="11" t="n"/>
+      <c r="AB9" s="11" t="n"/>
+      <c r="AC9" s="11" t="n"/>
+      <c r="AD9" s="11" t="n"/>
+      <c r="AE9" s="11" t="n"/>
+      <c r="AF9" s="11" t="n"/>
+      <c r="AG9" s="11" t="n"/>
+      <c r="AH9" s="11" t="n"/>
+      <c r="AI9" s="11" t="n"/>
+      <c r="AJ9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -40250,6 +40689,35 @@
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="n"/>
+      <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="11" t="n"/>
+      <c r="R10" s="11" t="n"/>
+      <c r="S10" s="11" t="n"/>
+      <c r="T10" s="11" t="n"/>
+      <c r="U10" s="11" t="n"/>
+      <c r="V10" s="11" t="n"/>
+      <c r="W10" s="11" t="n"/>
+      <c r="X10" s="11" t="n"/>
+      <c r="Y10" s="11" t="n"/>
+      <c r="Z10" s="11" t="n"/>
+      <c r="AA10" s="11" t="n"/>
+      <c r="AB10" s="11" t="n"/>
+      <c r="AC10" s="11" t="n"/>
+      <c r="AD10" s="11" t="n"/>
+      <c r="AE10" s="11" t="n"/>
+      <c r="AF10" s="11" t="n"/>
+      <c r="AG10" s="11" t="n"/>
+      <c r="AH10" s="11" t="n"/>
+      <c r="AI10" s="11" t="n"/>
+      <c r="AJ10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -40303,6 +40771,35 @@
           <t>Modest efficacy vs Dupixent</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>遞交</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="n"/>
+      <c r="O11" s="13" t="n"/>
+      <c r="P11" s="13" t="n"/>
+      <c r="Q11" s="11" t="n"/>
+      <c r="R11" s="11" t="n"/>
+      <c r="S11" s="11" t="n"/>
+      <c r="T11" s="11" t="n"/>
+      <c r="U11" s="11" t="n"/>
+      <c r="V11" s="11" t="n"/>
+      <c r="W11" s="11" t="n"/>
+      <c r="X11" s="11" t="n"/>
+      <c r="Y11" s="11" t="n"/>
+      <c r="Z11" s="11" t="n"/>
+      <c r="AA11" s="11" t="n"/>
+      <c r="AB11" s="11" t="n"/>
+      <c r="AC11" s="11" t="n"/>
+      <c r="AD11" s="11" t="n"/>
+      <c r="AE11" s="11" t="n"/>
+      <c r="AF11" s="11" t="n"/>
+      <c r="AG11" s="11" t="n"/>
+      <c r="AH11" s="11" t="n"/>
+      <c r="AI11" s="11" t="n"/>
+      <c r="AJ11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -40356,6 +40853,35 @@
           <t>Partner: Arcellx (ACLX)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N12" s="10" t="n"/>
+      <c r="O12" s="10" t="n"/>
+      <c r="P12" s="10" t="n"/>
+      <c r="Q12" s="11" t="n"/>
+      <c r="R12" s="11" t="n"/>
+      <c r="S12" s="11" t="n"/>
+      <c r="T12" s="11" t="n"/>
+      <c r="U12" s="11" t="n"/>
+      <c r="V12" s="11" t="n"/>
+      <c r="W12" s="11" t="n"/>
+      <c r="X12" s="11" t="n"/>
+      <c r="Y12" s="11" t="n"/>
+      <c r="Z12" s="11" t="n"/>
+      <c r="AA12" s="11" t="n"/>
+      <c r="AB12" s="11" t="n"/>
+      <c r="AC12" s="11" t="n"/>
+      <c r="AD12" s="11" t="n"/>
+      <c r="AE12" s="11" t="n"/>
+      <c r="AF12" s="11" t="n"/>
+      <c r="AG12" s="11" t="n"/>
+      <c r="AH12" s="11" t="n"/>
+      <c r="AI12" s="11" t="n"/>
+      <c r="AJ12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -40405,6 +40931,35 @@
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="n"/>
+      <c r="O13" s="10" t="n"/>
+      <c r="P13" s="10" t="n"/>
+      <c r="Q13" s="11" t="n"/>
+      <c r="R13" s="11" t="n"/>
+      <c r="S13" s="11" t="n"/>
+      <c r="T13" s="11" t="n"/>
+      <c r="U13" s="11" t="n"/>
+      <c r="V13" s="11" t="n"/>
+      <c r="W13" s="11" t="n"/>
+      <c r="X13" s="11" t="n"/>
+      <c r="Y13" s="11" t="n"/>
+      <c r="Z13" s="11" t="n"/>
+      <c r="AA13" s="11" t="n"/>
+      <c r="AB13" s="11" t="n"/>
+      <c r="AC13" s="11" t="n"/>
+      <c r="AD13" s="11" t="n"/>
+      <c r="AE13" s="11" t="n"/>
+      <c r="AF13" s="11" t="n"/>
+      <c r="AG13" s="11" t="n"/>
+      <c r="AH13" s="11" t="n"/>
+      <c r="AI13" s="11" t="n"/>
+      <c r="AJ13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -40454,6 +41009,35 @@
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: 事件</t>
+        </is>
+      </c>
+      <c r="M14" s="11" t="n"/>
+      <c r="N14" s="11" t="n"/>
+      <c r="O14" s="11" t="n"/>
+      <c r="P14" s="11" t="n"/>
+      <c r="Q14" s="11" t="n"/>
+      <c r="R14" s="11" t="n"/>
+      <c r="S14" s="11" t="n"/>
+      <c r="T14" s="11" t="n"/>
+      <c r="U14" s="11" t="n"/>
+      <c r="V14" s="11" t="n"/>
+      <c r="W14" s="11" t="n"/>
+      <c r="X14" s="11" t="n"/>
+      <c r="Y14" s="11" t="n"/>
+      <c r="Z14" s="11" t="n"/>
+      <c r="AA14" s="11" t="n"/>
+      <c r="AB14" s="11" t="n"/>
+      <c r="AC14" s="11" t="n"/>
+      <c r="AD14" s="11" t="n"/>
+      <c r="AE14" s="11" t="n"/>
+      <c r="AF14" s="11" t="n"/>
+      <c r="AG14" s="11" t="n"/>
+      <c r="AH14" s="11" t="n"/>
+      <c r="AI14" s="11" t="n"/>
+      <c r="AJ14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -40503,6 +41087,35 @@
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>遞交</t>
+        </is>
+      </c>
+      <c r="N15" s="10" t="n"/>
+      <c r="O15" s="10" t="n"/>
+      <c r="P15" s="10" t="n"/>
+      <c r="Q15" s="11" t="n"/>
+      <c r="R15" s="11" t="n"/>
+      <c r="S15" s="11" t="n"/>
+      <c r="T15" s="11" t="n"/>
+      <c r="U15" s="11" t="n"/>
+      <c r="V15" s="11" t="n"/>
+      <c r="W15" s="11" t="n"/>
+      <c r="X15" s="11" t="n"/>
+      <c r="Y15" s="11" t="n"/>
+      <c r="Z15" s="11" t="n"/>
+      <c r="AA15" s="11" t="n"/>
+      <c r="AB15" s="11" t="n"/>
+      <c r="AC15" s="11" t="n"/>
+      <c r="AD15" s="11" t="n"/>
+      <c r="AE15" s="11" t="n"/>
+      <c r="AF15" s="11" t="n"/>
+      <c r="AG15" s="11" t="n"/>
+      <c r="AH15" s="11" t="n"/>
+      <c r="AI15" s="11" t="n"/>
+      <c r="AJ15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -40556,6 +41169,39 @@
           <t>~20-22% weight loss; below 25% target</t>
         </is>
       </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>逾期未發生: 遞交</t>
+        </is>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="n"/>
+      <c r="O16" s="13" t="n"/>
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="13" t="n"/>
+      <c r="R16" s="13" t="n"/>
+      <c r="S16" s="13" t="n"/>
+      <c r="T16" s="13" t="n"/>
+      <c r="U16" s="13" t="n"/>
+      <c r="V16" s="13" t="n"/>
+      <c r="W16" s="13" t="n"/>
+      <c r="X16" s="13" t="n"/>
+      <c r="Y16" s="13" t="n"/>
+      <c r="Z16" s="13" t="n"/>
+      <c r="AA16" s="13" t="n"/>
+      <c r="AB16" s="13" t="n"/>
+      <c r="AC16" s="11" t="n"/>
+      <c r="AD16" s="11" t="n"/>
+      <c r="AE16" s="11" t="n"/>
+      <c r="AF16" s="11" t="n"/>
+      <c r="AG16" s="11" t="n"/>
+      <c r="AH16" s="11" t="n"/>
+      <c r="AI16" s="11" t="n"/>
+      <c r="AJ16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -40605,6 +41251,35 @@
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="12" t="inlineStr">
+        <is>
+          <t>遞交</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="n"/>
+      <c r="O17" s="13" t="n"/>
+      <c r="P17" s="13" t="n"/>
+      <c r="Q17" s="11" t="n"/>
+      <c r="R17" s="11" t="n"/>
+      <c r="S17" s="11" t="n"/>
+      <c r="T17" s="11" t="n"/>
+      <c r="U17" s="11" t="n"/>
+      <c r="V17" s="11" t="n"/>
+      <c r="W17" s="11" t="n"/>
+      <c r="X17" s="11" t="n"/>
+      <c r="Y17" s="11" t="n"/>
+      <c r="Z17" s="11" t="n"/>
+      <c r="AA17" s="11" t="n"/>
+      <c r="AB17" s="11" t="n"/>
+      <c r="AC17" s="11" t="n"/>
+      <c r="AD17" s="11" t="n"/>
+      <c r="AE17" s="11" t="n"/>
+      <c r="AF17" s="11" t="n"/>
+      <c r="AG17" s="11" t="n"/>
+      <c r="AH17" s="11" t="n"/>
+      <c r="AI17" s="11" t="n"/>
+      <c r="AJ17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -40654,6 +41329,35 @@
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N18" s="10" t="n"/>
+      <c r="O18" s="10" t="n"/>
+      <c r="P18" s="10" t="n"/>
+      <c r="Q18" s="11" t="n"/>
+      <c r="R18" s="11" t="n"/>
+      <c r="S18" s="11" t="n"/>
+      <c r="T18" s="11" t="n"/>
+      <c r="U18" s="11" t="n"/>
+      <c r="V18" s="11" t="n"/>
+      <c r="W18" s="11" t="n"/>
+      <c r="X18" s="11" t="n"/>
+      <c r="Y18" s="11" t="n"/>
+      <c r="Z18" s="11" t="n"/>
+      <c r="AA18" s="11" t="n"/>
+      <c r="AB18" s="11" t="n"/>
+      <c r="AC18" s="11" t="n"/>
+      <c r="AD18" s="11" t="n"/>
+      <c r="AE18" s="11" t="n"/>
+      <c r="AF18" s="11" t="n"/>
+      <c r="AG18" s="11" t="n"/>
+      <c r="AH18" s="11" t="n"/>
+      <c r="AI18" s="11" t="n"/>
+      <c r="AJ18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -40703,6 +41407,35 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="n"/>
+      <c r="N19" s="11" t="n"/>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
+      <c r="Q19" s="11" t="n"/>
+      <c r="R19" s="11" t="n"/>
+      <c r="S19" s="11" t="n"/>
+      <c r="T19" s="11" t="n"/>
+      <c r="U19" s="11" t="n"/>
+      <c r="V19" s="11" t="n"/>
+      <c r="W19" s="11" t="n"/>
+      <c r="X19" s="11" t="n"/>
+      <c r="Y19" s="11" t="n"/>
+      <c r="Z19" s="11" t="n"/>
+      <c r="AA19" s="11" t="n"/>
+      <c r="AB19" s="11" t="n"/>
+      <c r="AC19" s="11" t="n"/>
+      <c r="AD19" s="11" t="n"/>
+      <c r="AE19" s="11" t="n"/>
+      <c r="AF19" s="11" t="n"/>
+      <c r="AG19" s="11" t="n"/>
+      <c r="AH19" s="11" t="n"/>
+      <c r="AI19" s="11" t="n"/>
+      <c r="AJ19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -40752,6 +41485,35 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>遞交</t>
+        </is>
+      </c>
+      <c r="N20" s="10" t="n"/>
+      <c r="O20" s="10" t="n"/>
+      <c r="P20" s="10" t="n"/>
+      <c r="Q20" s="11" t="n"/>
+      <c r="R20" s="11" t="n"/>
+      <c r="S20" s="11" t="n"/>
+      <c r="T20" s="11" t="n"/>
+      <c r="U20" s="11" t="n"/>
+      <c r="V20" s="11" t="n"/>
+      <c r="W20" s="11" t="n"/>
+      <c r="X20" s="11" t="n"/>
+      <c r="Y20" s="11" t="n"/>
+      <c r="Z20" s="11" t="n"/>
+      <c r="AA20" s="11" t="n"/>
+      <c r="AB20" s="11" t="n"/>
+      <c r="AC20" s="11" t="n"/>
+      <c r="AD20" s="11" t="n"/>
+      <c r="AE20" s="11" t="n"/>
+      <c r="AF20" s="11" t="n"/>
+      <c r="AG20" s="11" t="n"/>
+      <c r="AH20" s="11" t="n"/>
+      <c r="AI20" s="11" t="n"/>
+      <c r="AJ20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -40801,6 +41563,35 @@
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
+      <c r="Q21" s="11" t="n"/>
+      <c r="R21" s="11" t="n"/>
+      <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n"/>
+      <c r="U21" s="11" t="n"/>
+      <c r="V21" s="11" t="n"/>
+      <c r="W21" s="11" t="n"/>
+      <c r="X21" s="11" t="n"/>
+      <c r="Y21" s="11" t="n"/>
+      <c r="Z21" s="11" t="n"/>
+      <c r="AA21" s="11" t="n"/>
+      <c r="AB21" s="11" t="n"/>
+      <c r="AC21" s="11" t="n"/>
+      <c r="AD21" s="11" t="n"/>
+      <c r="AE21" s="11" t="n"/>
+      <c r="AF21" s="11" t="n"/>
+      <c r="AG21" s="11" t="n"/>
+      <c r="AH21" s="11" t="n"/>
+      <c r="AI21" s="11" t="n"/>
+      <c r="AJ21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -40850,6 +41641,35 @@
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="n"/>
+      <c r="O22" s="13" t="n"/>
+      <c r="P22" s="13" t="n"/>
+      <c r="Q22" s="11" t="n"/>
+      <c r="R22" s="11" t="n"/>
+      <c r="S22" s="11" t="n"/>
+      <c r="T22" s="11" t="n"/>
+      <c r="U22" s="11" t="n"/>
+      <c r="V22" s="11" t="n"/>
+      <c r="W22" s="11" t="n"/>
+      <c r="X22" s="11" t="n"/>
+      <c r="Y22" s="11" t="n"/>
+      <c r="Z22" s="11" t="n"/>
+      <c r="AA22" s="11" t="n"/>
+      <c r="AB22" s="11" t="n"/>
+      <c r="AC22" s="11" t="n"/>
+      <c r="AD22" s="11" t="n"/>
+      <c r="AE22" s="11" t="n"/>
+      <c r="AF22" s="11" t="n"/>
+      <c r="AG22" s="11" t="n"/>
+      <c r="AH22" s="11" t="n"/>
+      <c r="AI22" s="11" t="n"/>
+      <c r="AJ22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -40899,6 +41719,35 @@
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>遞交</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="n"/>
+      <c r="O23" s="10" t="n"/>
+      <c r="P23" s="10" t="n"/>
+      <c r="Q23" s="11" t="n"/>
+      <c r="R23" s="11" t="n"/>
+      <c r="S23" s="11" t="n"/>
+      <c r="T23" s="11" t="n"/>
+      <c r="U23" s="11" t="n"/>
+      <c r="V23" s="11" t="n"/>
+      <c r="W23" s="11" t="n"/>
+      <c r="X23" s="11" t="n"/>
+      <c r="Y23" s="11" t="n"/>
+      <c r="Z23" s="11" t="n"/>
+      <c r="AA23" s="11" t="n"/>
+      <c r="AB23" s="11" t="n"/>
+      <c r="AC23" s="11" t="n"/>
+      <c r="AD23" s="11" t="n"/>
+      <c r="AE23" s="11" t="n"/>
+      <c r="AF23" s="11" t="n"/>
+      <c r="AG23" s="11" t="n"/>
+      <c r="AH23" s="11" t="n"/>
+      <c r="AI23" s="11" t="n"/>
+      <c r="AJ23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -40952,6 +41801,35 @@
           <t>Liver safety concerns; regulatory uncertainty</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: 事件</t>
+        </is>
+      </c>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="n"/>
+      <c r="O24" s="11" t="n"/>
+      <c r="P24" s="11" t="n"/>
+      <c r="Q24" s="11" t="n"/>
+      <c r="R24" s="11" t="n"/>
+      <c r="S24" s="11" t="n"/>
+      <c r="T24" s="11" t="n"/>
+      <c r="U24" s="11" t="n"/>
+      <c r="V24" s="11" t="n"/>
+      <c r="W24" s="11" t="n"/>
+      <c r="X24" s="11" t="n"/>
+      <c r="Y24" s="11" t="n"/>
+      <c r="Z24" s="11" t="n"/>
+      <c r="AA24" s="11" t="n"/>
+      <c r="AB24" s="11" t="n"/>
+      <c r="AC24" s="11" t="n"/>
+      <c r="AD24" s="11" t="n"/>
+      <c r="AE24" s="11" t="n"/>
+      <c r="AF24" s="11" t="n"/>
+      <c r="AG24" s="11" t="n"/>
+      <c r="AH24" s="11" t="n"/>
+      <c r="AI24" s="11" t="n"/>
+      <c r="AJ24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -41001,6 +41879,35 @@
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M25" s="11" t="n"/>
+      <c r="N25" s="11" t="n"/>
+      <c r="O25" s="11" t="n"/>
+      <c r="P25" s="11" t="n"/>
+      <c r="Q25" s="11" t="n"/>
+      <c r="R25" s="11" t="n"/>
+      <c r="S25" s="11" t="n"/>
+      <c r="T25" s="11" t="n"/>
+      <c r="U25" s="11" t="n"/>
+      <c r="V25" s="11" t="n"/>
+      <c r="W25" s="11" t="n"/>
+      <c r="X25" s="11" t="n"/>
+      <c r="Y25" s="11" t="n"/>
+      <c r="Z25" s="11" t="n"/>
+      <c r="AA25" s="11" t="n"/>
+      <c r="AB25" s="11" t="n"/>
+      <c r="AC25" s="11" t="n"/>
+      <c r="AD25" s="11" t="n"/>
+      <c r="AE25" s="11" t="n"/>
+      <c r="AF25" s="11" t="n"/>
+      <c r="AG25" s="11" t="n"/>
+      <c r="AH25" s="11" t="n"/>
+      <c r="AI25" s="11" t="n"/>
+      <c r="AJ25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -41050,6 +41957,35 @@
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N26" s="10" t="n"/>
+      <c r="O26" s="10" t="n"/>
+      <c r="P26" s="10" t="n"/>
+      <c r="Q26" s="11" t="n"/>
+      <c r="R26" s="11" t="n"/>
+      <c r="S26" s="11" t="n"/>
+      <c r="T26" s="11" t="n"/>
+      <c r="U26" s="11" t="n"/>
+      <c r="V26" s="11" t="n"/>
+      <c r="W26" s="11" t="n"/>
+      <c r="X26" s="11" t="n"/>
+      <c r="Y26" s="11" t="n"/>
+      <c r="Z26" s="11" t="n"/>
+      <c r="AA26" s="11" t="n"/>
+      <c r="AB26" s="11" t="n"/>
+      <c r="AC26" s="11" t="n"/>
+      <c r="AD26" s="11" t="n"/>
+      <c r="AE26" s="11" t="n"/>
+      <c r="AF26" s="11" t="n"/>
+      <c r="AG26" s="11" t="n"/>
+      <c r="AH26" s="11" t="n"/>
+      <c r="AI26" s="11" t="n"/>
+      <c r="AJ26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -41103,6 +42039,35 @@
           <t>First-in-class orexin agonist</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="n"/>
+      <c r="O27" s="10" t="n"/>
+      <c r="P27" s="10" t="n"/>
+      <c r="Q27" s="11" t="n"/>
+      <c r="R27" s="11" t="n"/>
+      <c r="S27" s="11" t="n"/>
+      <c r="T27" s="11" t="n"/>
+      <c r="U27" s="11" t="n"/>
+      <c r="V27" s="11" t="n"/>
+      <c r="W27" s="11" t="n"/>
+      <c r="X27" s="11" t="n"/>
+      <c r="Y27" s="11" t="n"/>
+      <c r="Z27" s="11" t="n"/>
+      <c r="AA27" s="11" t="n"/>
+      <c r="AB27" s="11" t="n"/>
+      <c r="AC27" s="11" t="n"/>
+      <c r="AD27" s="11" t="n"/>
+      <c r="AE27" s="11" t="n"/>
+      <c r="AF27" s="11" t="n"/>
+      <c r="AG27" s="11" t="n"/>
+      <c r="AH27" s="11" t="n"/>
+      <c r="AI27" s="11" t="n"/>
+      <c r="AJ27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -41156,6 +42121,35 @@
           <t>Partner Protagonist (PTGX)</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M28" s="11" t="n"/>
+      <c r="N28" s="11" t="n"/>
+      <c r="O28" s="11" t="n"/>
+      <c r="P28" s="11" t="n"/>
+      <c r="Q28" s="11" t="n"/>
+      <c r="R28" s="11" t="n"/>
+      <c r="S28" s="11" t="n"/>
+      <c r="T28" s="11" t="n"/>
+      <c r="U28" s="11" t="n"/>
+      <c r="V28" s="11" t="n"/>
+      <c r="W28" s="11" t="n"/>
+      <c r="X28" s="11" t="n"/>
+      <c r="Y28" s="11" t="n"/>
+      <c r="Z28" s="11" t="n"/>
+      <c r="AA28" s="11" t="n"/>
+      <c r="AB28" s="11" t="n"/>
+      <c r="AC28" s="11" t="n"/>
+      <c r="AD28" s="11" t="n"/>
+      <c r="AE28" s="11" t="n"/>
+      <c r="AF28" s="11" t="n"/>
+      <c r="AG28" s="11" t="n"/>
+      <c r="AH28" s="11" t="n"/>
+      <c r="AI28" s="11" t="n"/>
+      <c r="AJ28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -41205,6 +42199,35 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M29" s="11" t="n"/>
+      <c r="N29" s="11" t="n"/>
+      <c r="O29" s="11" t="n"/>
+      <c r="P29" s="11" t="n"/>
+      <c r="Q29" s="11" t="n"/>
+      <c r="R29" s="11" t="n"/>
+      <c r="S29" s="11" t="n"/>
+      <c r="T29" s="11" t="n"/>
+      <c r="U29" s="11" t="n"/>
+      <c r="V29" s="11" t="n"/>
+      <c r="W29" s="11" t="n"/>
+      <c r="X29" s="11" t="n"/>
+      <c r="Y29" s="11" t="n"/>
+      <c r="Z29" s="11" t="n"/>
+      <c r="AA29" s="11" t="n"/>
+      <c r="AB29" s="11" t="n"/>
+      <c r="AC29" s="11" t="n"/>
+      <c r="AD29" s="11" t="n"/>
+      <c r="AE29" s="11" t="n"/>
+      <c r="AF29" s="11" t="n"/>
+      <c r="AG29" s="11" t="n"/>
+      <c r="AH29" s="11" t="n"/>
+      <c r="AI29" s="11" t="n"/>
+      <c r="AJ29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -41254,6 +42277,35 @@
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: 事件</t>
+        </is>
+      </c>
+      <c r="M30" s="11" t="n"/>
+      <c r="N30" s="11" t="n"/>
+      <c r="O30" s="11" t="n"/>
+      <c r="P30" s="11" t="n"/>
+      <c r="Q30" s="11" t="n"/>
+      <c r="R30" s="11" t="n"/>
+      <c r="S30" s="11" t="n"/>
+      <c r="T30" s="11" t="n"/>
+      <c r="U30" s="11" t="n"/>
+      <c r="V30" s="11" t="n"/>
+      <c r="W30" s="11" t="n"/>
+      <c r="X30" s="11" t="n"/>
+      <c r="Y30" s="11" t="n"/>
+      <c r="Z30" s="11" t="n"/>
+      <c r="AA30" s="11" t="n"/>
+      <c r="AB30" s="11" t="n"/>
+      <c r="AC30" s="11" t="n"/>
+      <c r="AD30" s="11" t="n"/>
+      <c r="AE30" s="11" t="n"/>
+      <c r="AF30" s="11" t="n"/>
+      <c r="AG30" s="11" t="n"/>
+      <c r="AH30" s="11" t="n"/>
+      <c r="AI30" s="11" t="n"/>
+      <c r="AJ30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -41307,6 +42359,35 @@
           <t>Partner AstraZeneca</t>
         </is>
       </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N31" s="10" t="n"/>
+      <c r="O31" s="10" t="n"/>
+      <c r="P31" s="10" t="n"/>
+      <c r="Q31" s="11" t="n"/>
+      <c r="R31" s="11" t="n"/>
+      <c r="S31" s="11" t="n"/>
+      <c r="T31" s="11" t="n"/>
+      <c r="U31" s="11" t="n"/>
+      <c r="V31" s="11" t="n"/>
+      <c r="W31" s="11" t="n"/>
+      <c r="X31" s="11" t="n"/>
+      <c r="Y31" s="11" t="n"/>
+      <c r="Z31" s="11" t="n"/>
+      <c r="AA31" s="11" t="n"/>
+      <c r="AB31" s="11" t="n"/>
+      <c r="AC31" s="11" t="n"/>
+      <c r="AD31" s="11" t="n"/>
+      <c r="AE31" s="11" t="n"/>
+      <c r="AF31" s="11" t="n"/>
+      <c r="AG31" s="11" t="n"/>
+      <c r="AH31" s="11" t="n"/>
+      <c r="AI31" s="11" t="n"/>
+      <c r="AJ31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -41360,6 +42441,35 @@
           <t>OS immaturity is key FDA risk</t>
         </is>
       </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="12" t="inlineStr">
+        <is>
+          <t>事件</t>
+        </is>
+      </c>
+      <c r="N32" s="13" t="n"/>
+      <c r="O32" s="13" t="n"/>
+      <c r="P32" s="13" t="n"/>
+      <c r="Q32" s="13" t="n"/>
+      <c r="R32" s="13" t="n"/>
+      <c r="S32" s="13" t="n"/>
+      <c r="T32" s="13" t="n"/>
+      <c r="U32" s="13" t="n"/>
+      <c r="V32" s="13" t="n"/>
+      <c r="W32" s="13" t="n"/>
+      <c r="X32" s="13" t="n"/>
+      <c r="Y32" s="13" t="n"/>
+      <c r="Z32" s="13" t="n"/>
+      <c r="AA32" s="13" t="n"/>
+      <c r="AB32" s="13" t="n"/>
+      <c r="AC32" s="11" t="n"/>
+      <c r="AD32" s="11" t="n"/>
+      <c r="AE32" s="11" t="n"/>
+      <c r="AF32" s="11" t="n"/>
+      <c r="AG32" s="11" t="n"/>
+      <c r="AH32" s="11" t="n"/>
+      <c r="AI32" s="11" t="n"/>
+      <c r="AJ32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -41409,6 +42519,35 @@
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N33" s="10" t="n"/>
+      <c r="O33" s="10" t="n"/>
+      <c r="P33" s="10" t="n"/>
+      <c r="Q33" s="11" t="n"/>
+      <c r="R33" s="11" t="n"/>
+      <c r="S33" s="11" t="n"/>
+      <c r="T33" s="11" t="n"/>
+      <c r="U33" s="11" t="n"/>
+      <c r="V33" s="11" t="n"/>
+      <c r="W33" s="11" t="n"/>
+      <c r="X33" s="11" t="n"/>
+      <c r="Y33" s="11" t="n"/>
+      <c r="Z33" s="11" t="n"/>
+      <c r="AA33" s="11" t="n"/>
+      <c r="AB33" s="11" t="n"/>
+      <c r="AC33" s="11" t="n"/>
+      <c r="AD33" s="11" t="n"/>
+      <c r="AE33" s="11" t="n"/>
+      <c r="AF33" s="11" t="n"/>
+      <c r="AG33" s="11" t="n"/>
+      <c r="AH33" s="11" t="n"/>
+      <c r="AI33" s="11" t="n"/>
+      <c r="AJ33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -41458,6 +42597,35 @@
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N34" s="10" t="n"/>
+      <c r="O34" s="10" t="n"/>
+      <c r="P34" s="10" t="n"/>
+      <c r="Q34" s="11" t="n"/>
+      <c r="R34" s="11" t="n"/>
+      <c r="S34" s="11" t="n"/>
+      <c r="T34" s="11" t="n"/>
+      <c r="U34" s="11" t="n"/>
+      <c r="V34" s="11" t="n"/>
+      <c r="W34" s="11" t="n"/>
+      <c r="X34" s="11" t="n"/>
+      <c r="Y34" s="11" t="n"/>
+      <c r="Z34" s="11" t="n"/>
+      <c r="AA34" s="11" t="n"/>
+      <c r="AB34" s="11" t="n"/>
+      <c r="AC34" s="11" t="n"/>
+      <c r="AD34" s="11" t="n"/>
+      <c r="AE34" s="11" t="n"/>
+      <c r="AF34" s="11" t="n"/>
+      <c r="AG34" s="11" t="n"/>
+      <c r="AH34" s="11" t="n"/>
+      <c r="AI34" s="11" t="n"/>
+      <c r="AJ34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -41511,6 +42679,35 @@
           <t>One of three Ph3 missed</t>
         </is>
       </c>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N35" s="10" t="n"/>
+      <c r="O35" s="10" t="n"/>
+      <c r="P35" s="10" t="n"/>
+      <c r="Q35" s="11" t="n"/>
+      <c r="R35" s="11" t="n"/>
+      <c r="S35" s="11" t="n"/>
+      <c r="T35" s="11" t="n"/>
+      <c r="U35" s="11" t="n"/>
+      <c r="V35" s="11" t="n"/>
+      <c r="W35" s="11" t="n"/>
+      <c r="X35" s="11" t="n"/>
+      <c r="Y35" s="11" t="n"/>
+      <c r="Z35" s="11" t="n"/>
+      <c r="AA35" s="11" t="n"/>
+      <c r="AB35" s="11" t="n"/>
+      <c r="AC35" s="11" t="n"/>
+      <c r="AD35" s="11" t="n"/>
+      <c r="AE35" s="11" t="n"/>
+      <c r="AF35" s="11" t="n"/>
+      <c r="AG35" s="11" t="n"/>
+      <c r="AH35" s="11" t="n"/>
+      <c r="AI35" s="11" t="n"/>
+      <c r="AJ35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -41560,6 +42757,35 @@
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M36" s="11" t="n"/>
+      <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11" t="n"/>
+      <c r="P36" s="11" t="n"/>
+      <c r="Q36" s="11" t="n"/>
+      <c r="R36" s="11" t="n"/>
+      <c r="S36" s="11" t="n"/>
+      <c r="T36" s="11" t="n"/>
+      <c r="U36" s="11" t="n"/>
+      <c r="V36" s="11" t="n"/>
+      <c r="W36" s="11" t="n"/>
+      <c r="X36" s="11" t="n"/>
+      <c r="Y36" s="11" t="n"/>
+      <c r="Z36" s="11" t="n"/>
+      <c r="AA36" s="11" t="n"/>
+      <c r="AB36" s="11" t="n"/>
+      <c r="AC36" s="11" t="n"/>
+      <c r="AD36" s="11" t="n"/>
+      <c r="AE36" s="11" t="n"/>
+      <c r="AF36" s="11" t="n"/>
+      <c r="AG36" s="11" t="n"/>
+      <c r="AH36" s="11" t="n"/>
+      <c r="AI36" s="11" t="n"/>
+      <c r="AJ36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -41609,6 +42835,35 @@
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="12" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N37" s="13" t="n"/>
+      <c r="O37" s="13" t="n"/>
+      <c r="P37" s="13" t="n"/>
+      <c r="Q37" s="11" t="n"/>
+      <c r="R37" s="11" t="n"/>
+      <c r="S37" s="11" t="n"/>
+      <c r="T37" s="11" t="n"/>
+      <c r="U37" s="11" t="n"/>
+      <c r="V37" s="11" t="n"/>
+      <c r="W37" s="11" t="n"/>
+      <c r="X37" s="11" t="n"/>
+      <c r="Y37" s="11" t="n"/>
+      <c r="Z37" s="11" t="n"/>
+      <c r="AA37" s="11" t="n"/>
+      <c r="AB37" s="11" t="n"/>
+      <c r="AC37" s="11" t="n"/>
+      <c r="AD37" s="11" t="n"/>
+      <c r="AE37" s="11" t="n"/>
+      <c r="AF37" s="11" t="n"/>
+      <c r="AG37" s="11" t="n"/>
+      <c r="AH37" s="11" t="n"/>
+      <c r="AI37" s="11" t="n"/>
+      <c r="AJ37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -41658,6 +42913,35 @@
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N38" s="10" t="n"/>
+      <c r="O38" s="10" t="n"/>
+      <c r="P38" s="10" t="n"/>
+      <c r="Q38" s="11" t="n"/>
+      <c r="R38" s="11" t="n"/>
+      <c r="S38" s="11" t="n"/>
+      <c r="T38" s="11" t="n"/>
+      <c r="U38" s="11" t="n"/>
+      <c r="V38" s="11" t="n"/>
+      <c r="W38" s="11" t="n"/>
+      <c r="X38" s="11" t="n"/>
+      <c r="Y38" s="11" t="n"/>
+      <c r="Z38" s="11" t="n"/>
+      <c r="AA38" s="11" t="n"/>
+      <c r="AB38" s="11" t="n"/>
+      <c r="AC38" s="11" t="n"/>
+      <c r="AD38" s="11" t="n"/>
+      <c r="AE38" s="11" t="n"/>
+      <c r="AF38" s="11" t="n"/>
+      <c r="AG38" s="11" t="n"/>
+      <c r="AH38" s="11" t="n"/>
+      <c r="AI38" s="11" t="n"/>
+      <c r="AJ38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -41707,6 +42991,35 @@
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N39" s="10" t="n"/>
+      <c r="O39" s="10" t="n"/>
+      <c r="P39" s="10" t="n"/>
+      <c r="Q39" s="11" t="n"/>
+      <c r="R39" s="11" t="n"/>
+      <c r="S39" s="11" t="n"/>
+      <c r="T39" s="11" t="n"/>
+      <c r="U39" s="11" t="n"/>
+      <c r="V39" s="11" t="n"/>
+      <c r="W39" s="11" t="n"/>
+      <c r="X39" s="11" t="n"/>
+      <c r="Y39" s="11" t="n"/>
+      <c r="Z39" s="11" t="n"/>
+      <c r="AA39" s="11" t="n"/>
+      <c r="AB39" s="11" t="n"/>
+      <c r="AC39" s="11" t="n"/>
+      <c r="AD39" s="11" t="n"/>
+      <c r="AE39" s="11" t="n"/>
+      <c r="AF39" s="11" t="n"/>
+      <c r="AG39" s="11" t="n"/>
+      <c r="AH39" s="11" t="n"/>
+      <c r="AI39" s="11" t="n"/>
+      <c r="AJ39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -41756,6 +43069,35 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N40" s="10" t="n"/>
+      <c r="O40" s="10" t="n"/>
+      <c r="P40" s="10" t="n"/>
+      <c r="Q40" s="11" t="n"/>
+      <c r="R40" s="11" t="n"/>
+      <c r="S40" s="11" t="n"/>
+      <c r="T40" s="11" t="n"/>
+      <c r="U40" s="11" t="n"/>
+      <c r="V40" s="11" t="n"/>
+      <c r="W40" s="11" t="n"/>
+      <c r="X40" s="11" t="n"/>
+      <c r="Y40" s="11" t="n"/>
+      <c r="Z40" s="11" t="n"/>
+      <c r="AA40" s="11" t="n"/>
+      <c r="AB40" s="11" t="n"/>
+      <c r="AC40" s="11" t="n"/>
+      <c r="AD40" s="11" t="n"/>
+      <c r="AE40" s="11" t="n"/>
+      <c r="AF40" s="11" t="n"/>
+      <c r="AG40" s="11" t="n"/>
+      <c r="AH40" s="11" t="n"/>
+      <c r="AI40" s="11" t="n"/>
+      <c r="AJ40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -41805,6 +43147,35 @@
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N41" s="10" t="n"/>
+      <c r="O41" s="10" t="n"/>
+      <c r="P41" s="10" t="n"/>
+      <c r="Q41" s="11" t="n"/>
+      <c r="R41" s="11" t="n"/>
+      <c r="S41" s="11" t="n"/>
+      <c r="T41" s="11" t="n"/>
+      <c r="U41" s="11" t="n"/>
+      <c r="V41" s="11" t="n"/>
+      <c r="W41" s="11" t="n"/>
+      <c r="X41" s="11" t="n"/>
+      <c r="Y41" s="11" t="n"/>
+      <c r="Z41" s="11" t="n"/>
+      <c r="AA41" s="11" t="n"/>
+      <c r="AB41" s="11" t="n"/>
+      <c r="AC41" s="11" t="n"/>
+      <c r="AD41" s="11" t="n"/>
+      <c r="AE41" s="11" t="n"/>
+      <c r="AF41" s="11" t="n"/>
+      <c r="AG41" s="11" t="n"/>
+      <c r="AH41" s="11" t="n"/>
+      <c r="AI41" s="11" t="n"/>
+      <c r="AJ41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -41854,6 +43225,35 @@
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M42" s="11" t="n"/>
+      <c r="N42" s="11" t="n"/>
+      <c r="O42" s="11" t="n"/>
+      <c r="P42" s="11" t="n"/>
+      <c r="Q42" s="11" t="n"/>
+      <c r="R42" s="11" t="n"/>
+      <c r="S42" s="11" t="n"/>
+      <c r="T42" s="11" t="n"/>
+      <c r="U42" s="11" t="n"/>
+      <c r="V42" s="11" t="n"/>
+      <c r="W42" s="11" t="n"/>
+      <c r="X42" s="11" t="n"/>
+      <c r="Y42" s="11" t="n"/>
+      <c r="Z42" s="11" t="n"/>
+      <c r="AA42" s="11" t="n"/>
+      <c r="AB42" s="11" t="n"/>
+      <c r="AC42" s="11" t="n"/>
+      <c r="AD42" s="11" t="n"/>
+      <c r="AE42" s="11" t="n"/>
+      <c r="AF42" s="11" t="n"/>
+      <c r="AG42" s="11" t="n"/>
+      <c r="AH42" s="11" t="n"/>
+      <c r="AI42" s="11" t="n"/>
+      <c r="AJ42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -41907,6 +43307,35 @@
           <t>FDA vaccine policy uncertainty</t>
         </is>
       </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: BLA</t>
+        </is>
+      </c>
+      <c r="M43" s="11" t="n"/>
+      <c r="N43" s="11" t="n"/>
+      <c r="O43" s="11" t="n"/>
+      <c r="P43" s="11" t="n"/>
+      <c r="Q43" s="11" t="n"/>
+      <c r="R43" s="11" t="n"/>
+      <c r="S43" s="11" t="n"/>
+      <c r="T43" s="11" t="n"/>
+      <c r="U43" s="11" t="n"/>
+      <c r="V43" s="11" t="n"/>
+      <c r="W43" s="11" t="n"/>
+      <c r="X43" s="11" t="n"/>
+      <c r="Y43" s="11" t="n"/>
+      <c r="Z43" s="11" t="n"/>
+      <c r="AA43" s="11" t="n"/>
+      <c r="AB43" s="11" t="n"/>
+      <c r="AC43" s="11" t="n"/>
+      <c r="AD43" s="11" t="n"/>
+      <c r="AE43" s="11" t="n"/>
+      <c r="AF43" s="11" t="n"/>
+      <c r="AG43" s="11" t="n"/>
+      <c r="AH43" s="11" t="n"/>
+      <c r="AI43" s="11" t="n"/>
+      <c r="AJ43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -41956,6 +43385,35 @@
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M44" s="11" t="n"/>
+      <c r="N44" s="11" t="n"/>
+      <c r="O44" s="11" t="n"/>
+      <c r="P44" s="11" t="n"/>
+      <c r="Q44" s="11" t="n"/>
+      <c r="R44" s="11" t="n"/>
+      <c r="S44" s="11" t="n"/>
+      <c r="T44" s="11" t="n"/>
+      <c r="U44" s="11" t="n"/>
+      <c r="V44" s="11" t="n"/>
+      <c r="W44" s="11" t="n"/>
+      <c r="X44" s="11" t="n"/>
+      <c r="Y44" s="11" t="n"/>
+      <c r="Z44" s="11" t="n"/>
+      <c r="AA44" s="11" t="n"/>
+      <c r="AB44" s="11" t="n"/>
+      <c r="AC44" s="11" t="n"/>
+      <c r="AD44" s="11" t="n"/>
+      <c r="AE44" s="11" t="n"/>
+      <c r="AF44" s="11" t="n"/>
+      <c r="AG44" s="11" t="n"/>
+      <c r="AH44" s="11" t="n"/>
+      <c r="AI44" s="11" t="n"/>
+      <c r="AJ44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -42009,6 +43467,35 @@
           <t>Seeking commercialization partner</t>
         </is>
       </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M45" s="11" t="n"/>
+      <c r="N45" s="11" t="n"/>
+      <c r="O45" s="11" t="n"/>
+      <c r="P45" s="11" t="n"/>
+      <c r="Q45" s="11" t="n"/>
+      <c r="R45" s="11" t="n"/>
+      <c r="S45" s="11" t="n"/>
+      <c r="T45" s="11" t="n"/>
+      <c r="U45" s="11" t="n"/>
+      <c r="V45" s="11" t="n"/>
+      <c r="W45" s="11" t="n"/>
+      <c r="X45" s="11" t="n"/>
+      <c r="Y45" s="11" t="n"/>
+      <c r="Z45" s="11" t="n"/>
+      <c r="AA45" s="11" t="n"/>
+      <c r="AB45" s="11" t="n"/>
+      <c r="AC45" s="11" t="n"/>
+      <c r="AD45" s="11" t="n"/>
+      <c r="AE45" s="11" t="n"/>
+      <c r="AF45" s="11" t="n"/>
+      <c r="AG45" s="11" t="n"/>
+      <c r="AH45" s="11" t="n"/>
+      <c r="AI45" s="11" t="n"/>
+      <c r="AJ45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -42058,6 +43545,35 @@
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N46" s="10" t="n"/>
+      <c r="O46" s="10" t="n"/>
+      <c r="P46" s="10" t="n"/>
+      <c r="Q46" s="11" t="n"/>
+      <c r="R46" s="11" t="n"/>
+      <c r="S46" s="11" t="n"/>
+      <c r="T46" s="11" t="n"/>
+      <c r="U46" s="11" t="n"/>
+      <c r="V46" s="11" t="n"/>
+      <c r="W46" s="11" t="n"/>
+      <c r="X46" s="11" t="n"/>
+      <c r="Y46" s="11" t="n"/>
+      <c r="Z46" s="11" t="n"/>
+      <c r="AA46" s="11" t="n"/>
+      <c r="AB46" s="11" t="n"/>
+      <c r="AC46" s="11" t="n"/>
+      <c r="AD46" s="11" t="n"/>
+      <c r="AE46" s="11" t="n"/>
+      <c r="AF46" s="11" t="n"/>
+      <c r="AG46" s="11" t="n"/>
+      <c r="AH46" s="11" t="n"/>
+      <c r="AI46" s="11" t="n"/>
+      <c r="AJ46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -42107,6 +43623,35 @@
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N47" s="10" t="n"/>
+      <c r="O47" s="10" t="n"/>
+      <c r="P47" s="10" t="n"/>
+      <c r="Q47" s="11" t="n"/>
+      <c r="R47" s="11" t="n"/>
+      <c r="S47" s="11" t="n"/>
+      <c r="T47" s="11" t="n"/>
+      <c r="U47" s="11" t="n"/>
+      <c r="V47" s="11" t="n"/>
+      <c r="W47" s="11" t="n"/>
+      <c r="X47" s="11" t="n"/>
+      <c r="Y47" s="11" t="n"/>
+      <c r="Z47" s="11" t="n"/>
+      <c r="AA47" s="11" t="n"/>
+      <c r="AB47" s="11" t="n"/>
+      <c r="AC47" s="11" t="n"/>
+      <c r="AD47" s="11" t="n"/>
+      <c r="AE47" s="11" t="n"/>
+      <c r="AF47" s="11" t="n"/>
+      <c r="AG47" s="11" t="n"/>
+      <c r="AH47" s="11" t="n"/>
+      <c r="AI47" s="11" t="n"/>
+      <c r="AJ47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -42156,6 +43701,35 @@
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: PDUFA</t>
+        </is>
+      </c>
+      <c r="M48" s="11" t="n"/>
+      <c r="N48" s="11" t="n"/>
+      <c r="O48" s="11" t="n"/>
+      <c r="P48" s="11" t="n"/>
+      <c r="Q48" s="11" t="n"/>
+      <c r="R48" s="11" t="n"/>
+      <c r="S48" s="11" t="n"/>
+      <c r="T48" s="11" t="n"/>
+      <c r="U48" s="11" t="n"/>
+      <c r="V48" s="11" t="n"/>
+      <c r="W48" s="11" t="n"/>
+      <c r="X48" s="11" t="n"/>
+      <c r="Y48" s="11" t="n"/>
+      <c r="Z48" s="11" t="n"/>
+      <c r="AA48" s="11" t="n"/>
+      <c r="AB48" s="11" t="n"/>
+      <c r="AC48" s="11" t="n"/>
+      <c r="AD48" s="11" t="n"/>
+      <c r="AE48" s="11" t="n"/>
+      <c r="AF48" s="11" t="n"/>
+      <c r="AG48" s="11" t="n"/>
+      <c r="AH48" s="11" t="n"/>
+      <c r="AI48" s="11" t="n"/>
+      <c r="AJ48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -42209,6 +43783,35 @@
           <t>Accelerated approval on CSF HS biomarker</t>
         </is>
       </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M49" s="11" t="n"/>
+      <c r="N49" s="11" t="n"/>
+      <c r="O49" s="11" t="n"/>
+      <c r="P49" s="11" t="n"/>
+      <c r="Q49" s="11" t="n"/>
+      <c r="R49" s="11" t="n"/>
+      <c r="S49" s="11" t="n"/>
+      <c r="T49" s="11" t="n"/>
+      <c r="U49" s="11" t="n"/>
+      <c r="V49" s="11" t="n"/>
+      <c r="W49" s="11" t="n"/>
+      <c r="X49" s="11" t="n"/>
+      <c r="Y49" s="11" t="n"/>
+      <c r="Z49" s="11" t="n"/>
+      <c r="AA49" s="11" t="n"/>
+      <c r="AB49" s="11" t="n"/>
+      <c r="AC49" s="11" t="n"/>
+      <c r="AD49" s="11" t="n"/>
+      <c r="AE49" s="11" t="n"/>
+      <c r="AF49" s="11" t="n"/>
+      <c r="AG49" s="11" t="n"/>
+      <c r="AH49" s="11" t="n"/>
+      <c r="AI49" s="11" t="n"/>
+      <c r="AJ49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -42258,6 +43861,35 @@
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="10" t="n"/>
+      <c r="P50" s="10" t="n"/>
+      <c r="Q50" s="11" t="n"/>
+      <c r="R50" s="11" t="n"/>
+      <c r="S50" s="11" t="n"/>
+      <c r="T50" s="11" t="n"/>
+      <c r="U50" s="11" t="n"/>
+      <c r="V50" s="11" t="n"/>
+      <c r="W50" s="11" t="n"/>
+      <c r="X50" s="11" t="n"/>
+      <c r="Y50" s="11" t="n"/>
+      <c r="Z50" s="11" t="n"/>
+      <c r="AA50" s="11" t="n"/>
+      <c r="AB50" s="11" t="n"/>
+      <c r="AC50" s="11" t="n"/>
+      <c r="AD50" s="11" t="n"/>
+      <c r="AE50" s="11" t="n"/>
+      <c r="AF50" s="11" t="n"/>
+      <c r="AG50" s="11" t="n"/>
+      <c r="AH50" s="11" t="n"/>
+      <c r="AI50" s="11" t="n"/>
+      <c r="AJ50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -42307,6 +43939,35 @@
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="12" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N51" s="13" t="n"/>
+      <c r="O51" s="13" t="n"/>
+      <c r="P51" s="13" t="n"/>
+      <c r="Q51" s="11" t="n"/>
+      <c r="R51" s="11" t="n"/>
+      <c r="S51" s="11" t="n"/>
+      <c r="T51" s="11" t="n"/>
+      <c r="U51" s="11" t="n"/>
+      <c r="V51" s="11" t="n"/>
+      <c r="W51" s="11" t="n"/>
+      <c r="X51" s="11" t="n"/>
+      <c r="Y51" s="11" t="n"/>
+      <c r="Z51" s="11" t="n"/>
+      <c r="AA51" s="11" t="n"/>
+      <c r="AB51" s="11" t="n"/>
+      <c r="AC51" s="11" t="n"/>
+      <c r="AD51" s="11" t="n"/>
+      <c r="AE51" s="11" t="n"/>
+      <c r="AF51" s="11" t="n"/>
+      <c r="AG51" s="11" t="n"/>
+      <c r="AH51" s="11" t="n"/>
+      <c r="AI51" s="11" t="n"/>
+      <c r="AJ51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -42356,6 +44017,35 @@
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M52" s="11" t="n"/>
+      <c r="N52" s="11" t="n"/>
+      <c r="O52" s="11" t="n"/>
+      <c r="P52" s="11" t="n"/>
+      <c r="Q52" s="11" t="n"/>
+      <c r="R52" s="11" t="n"/>
+      <c r="S52" s="11" t="n"/>
+      <c r="T52" s="11" t="n"/>
+      <c r="U52" s="11" t="n"/>
+      <c r="V52" s="11" t="n"/>
+      <c r="W52" s="11" t="n"/>
+      <c r="X52" s="11" t="n"/>
+      <c r="Y52" s="11" t="n"/>
+      <c r="Z52" s="11" t="n"/>
+      <c r="AA52" s="11" t="n"/>
+      <c r="AB52" s="11" t="n"/>
+      <c r="AC52" s="11" t="n"/>
+      <c r="AD52" s="11" t="n"/>
+      <c r="AE52" s="11" t="n"/>
+      <c r="AF52" s="11" t="n"/>
+      <c r="AG52" s="11" t="n"/>
+      <c r="AH52" s="11" t="n"/>
+      <c r="AI52" s="11" t="n"/>
+      <c r="AJ52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -42405,6 +44095,35 @@
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N53" s="10" t="n"/>
+      <c r="O53" s="10" t="n"/>
+      <c r="P53" s="10" t="n"/>
+      <c r="Q53" s="11" t="n"/>
+      <c r="R53" s="11" t="n"/>
+      <c r="S53" s="11" t="n"/>
+      <c r="T53" s="11" t="n"/>
+      <c r="U53" s="11" t="n"/>
+      <c r="V53" s="11" t="n"/>
+      <c r="W53" s="11" t="n"/>
+      <c r="X53" s="11" t="n"/>
+      <c r="Y53" s="11" t="n"/>
+      <c r="Z53" s="11" t="n"/>
+      <c r="AA53" s="11" t="n"/>
+      <c r="AB53" s="11" t="n"/>
+      <c r="AC53" s="11" t="n"/>
+      <c r="AD53" s="11" t="n"/>
+      <c r="AE53" s="11" t="n"/>
+      <c r="AF53" s="11" t="n"/>
+      <c r="AG53" s="11" t="n"/>
+      <c r="AH53" s="11" t="n"/>
+      <c r="AI53" s="11" t="n"/>
+      <c r="AJ53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -42454,6 +44173,35 @@
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="15" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="N54" s="11" t="n"/>
+      <c r="O54" s="11" t="n"/>
+      <c r="P54" s="11" t="n"/>
+      <c r="Q54" s="11" t="n"/>
+      <c r="R54" s="11" t="n"/>
+      <c r="S54" s="11" t="n"/>
+      <c r="T54" s="11" t="n"/>
+      <c r="U54" s="11" t="n"/>
+      <c r="V54" s="11" t="n"/>
+      <c r="W54" s="11" t="n"/>
+      <c r="X54" s="11" t="n"/>
+      <c r="Y54" s="11" t="n"/>
+      <c r="Z54" s="11" t="n"/>
+      <c r="AA54" s="11" t="n"/>
+      <c r="AB54" s="11" t="n"/>
+      <c r="AC54" s="11" t="n"/>
+      <c r="AD54" s="11" t="n"/>
+      <c r="AE54" s="11" t="n"/>
+      <c r="AF54" s="11" t="n"/>
+      <c r="AG54" s="11" t="n"/>
+      <c r="AH54" s="11" t="n"/>
+      <c r="AI54" s="11" t="n"/>
+      <c r="AJ54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -42507,6 +44255,35 @@
           <t>Via Priovant</t>
         </is>
       </c>
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N55" s="10" t="n"/>
+      <c r="O55" s="10" t="n"/>
+      <c r="P55" s="10" t="n"/>
+      <c r="Q55" s="11" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="11" t="n"/>
+      <c r="T55" s="11" t="n"/>
+      <c r="U55" s="11" t="n"/>
+      <c r="V55" s="11" t="n"/>
+      <c r="W55" s="11" t="n"/>
+      <c r="X55" s="11" t="n"/>
+      <c r="Y55" s="11" t="n"/>
+      <c r="Z55" s="11" t="n"/>
+      <c r="AA55" s="11" t="n"/>
+      <c r="AB55" s="11" t="n"/>
+      <c r="AC55" s="11" t="n"/>
+      <c r="AD55" s="11" t="n"/>
+      <c r="AE55" s="11" t="n"/>
+      <c r="AF55" s="11" t="n"/>
+      <c r="AG55" s="11" t="n"/>
+      <c r="AH55" s="11" t="n"/>
+      <c r="AI55" s="11" t="n"/>
+      <c r="AJ55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -42560,6 +44337,35 @@
           <t>FDA priority voucher program</t>
         </is>
       </c>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="N56" s="10" t="n"/>
+      <c r="O56" s="10" t="n"/>
+      <c r="P56" s="10" t="n"/>
+      <c r="Q56" s="11" t="n"/>
+      <c r="R56" s="11" t="n"/>
+      <c r="S56" s="11" t="n"/>
+      <c r="T56" s="11" t="n"/>
+      <c r="U56" s="11" t="n"/>
+      <c r="V56" s="11" t="n"/>
+      <c r="W56" s="11" t="n"/>
+      <c r="X56" s="11" t="n"/>
+      <c r="Y56" s="11" t="n"/>
+      <c r="Z56" s="11" t="n"/>
+      <c r="AA56" s="11" t="n"/>
+      <c r="AB56" s="11" t="n"/>
+      <c r="AC56" s="11" t="n"/>
+      <c r="AD56" s="11" t="n"/>
+      <c r="AE56" s="11" t="n"/>
+      <c r="AF56" s="11" t="n"/>
+      <c r="AG56" s="11" t="n"/>
+      <c r="AH56" s="11" t="n"/>
+      <c r="AI56" s="11" t="n"/>
+      <c r="AJ56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -42613,6 +44419,35 @@
           <t>CRL due to manufacturing site (Catalent), not efficacy</t>
         </is>
       </c>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N57" s="10" t="n"/>
+      <c r="O57" s="10" t="n"/>
+      <c r="P57" s="10" t="n"/>
+      <c r="Q57" s="11" t="n"/>
+      <c r="R57" s="11" t="n"/>
+      <c r="S57" s="11" t="n"/>
+      <c r="T57" s="11" t="n"/>
+      <c r="U57" s="11" t="n"/>
+      <c r="V57" s="11" t="n"/>
+      <c r="W57" s="11" t="n"/>
+      <c r="X57" s="11" t="n"/>
+      <c r="Y57" s="11" t="n"/>
+      <c r="Z57" s="11" t="n"/>
+      <c r="AA57" s="11" t="n"/>
+      <c r="AB57" s="11" t="n"/>
+      <c r="AC57" s="11" t="n"/>
+      <c r="AD57" s="11" t="n"/>
+      <c r="AE57" s="11" t="n"/>
+      <c r="AF57" s="11" t="n"/>
+      <c r="AG57" s="11" t="n"/>
+      <c r="AH57" s="11" t="n"/>
+      <c r="AI57" s="11" t="n"/>
+      <c r="AJ57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -42662,6 +44497,35 @@
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M58" s="11" t="n"/>
+      <c r="N58" s="11" t="n"/>
+      <c r="O58" s="11" t="n"/>
+      <c r="P58" s="11" t="n"/>
+      <c r="Q58" s="11" t="n"/>
+      <c r="R58" s="11" t="n"/>
+      <c r="S58" s="11" t="n"/>
+      <c r="T58" s="11" t="n"/>
+      <c r="U58" s="11" t="n"/>
+      <c r="V58" s="11" t="n"/>
+      <c r="W58" s="11" t="n"/>
+      <c r="X58" s="11" t="n"/>
+      <c r="Y58" s="11" t="n"/>
+      <c r="Z58" s="11" t="n"/>
+      <c r="AA58" s="11" t="n"/>
+      <c r="AB58" s="11" t="n"/>
+      <c r="AC58" s="11" t="n"/>
+      <c r="AD58" s="11" t="n"/>
+      <c r="AE58" s="11" t="n"/>
+      <c r="AF58" s="11" t="n"/>
+      <c r="AG58" s="11" t="n"/>
+      <c r="AH58" s="11" t="n"/>
+      <c r="AI58" s="11" t="n"/>
+      <c r="AJ58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -42711,6 +44575,35 @@
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M59" s="11" t="n"/>
+      <c r="N59" s="11" t="n"/>
+      <c r="O59" s="11" t="n"/>
+      <c r="P59" s="11" t="n"/>
+      <c r="Q59" s="11" t="n"/>
+      <c r="R59" s="11" t="n"/>
+      <c r="S59" s="11" t="n"/>
+      <c r="T59" s="11" t="n"/>
+      <c r="U59" s="11" t="n"/>
+      <c r="V59" s="11" t="n"/>
+      <c r="W59" s="11" t="n"/>
+      <c r="X59" s="11" t="n"/>
+      <c r="Y59" s="11" t="n"/>
+      <c r="Z59" s="11" t="n"/>
+      <c r="AA59" s="11" t="n"/>
+      <c r="AB59" s="11" t="n"/>
+      <c r="AC59" s="11" t="n"/>
+      <c r="AD59" s="11" t="n"/>
+      <c r="AE59" s="11" t="n"/>
+      <c r="AF59" s="11" t="n"/>
+      <c r="AG59" s="11" t="n"/>
+      <c r="AH59" s="11" t="n"/>
+      <c r="AI59" s="11" t="n"/>
+      <c r="AJ59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -42760,6 +44653,35 @@
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N60" s="10" t="n"/>
+      <c r="O60" s="10" t="n"/>
+      <c r="P60" s="10" t="n"/>
+      <c r="Q60" s="11" t="n"/>
+      <c r="R60" s="11" t="n"/>
+      <c r="S60" s="11" t="n"/>
+      <c r="T60" s="11" t="n"/>
+      <c r="U60" s="11" t="n"/>
+      <c r="V60" s="11" t="n"/>
+      <c r="W60" s="11" t="n"/>
+      <c r="X60" s="11" t="n"/>
+      <c r="Y60" s="11" t="n"/>
+      <c r="Z60" s="11" t="n"/>
+      <c r="AA60" s="11" t="n"/>
+      <c r="AB60" s="11" t="n"/>
+      <c r="AC60" s="11" t="n"/>
+      <c r="AD60" s="11" t="n"/>
+      <c r="AE60" s="11" t="n"/>
+      <c r="AF60" s="11" t="n"/>
+      <c r="AG60" s="11" t="n"/>
+      <c r="AH60" s="11" t="n"/>
+      <c r="AI60" s="11" t="n"/>
+      <c r="AJ60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -42809,6 +44731,35 @@
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N61" s="10" t="n"/>
+      <c r="O61" s="10" t="n"/>
+      <c r="P61" s="10" t="n"/>
+      <c r="Q61" s="11" t="n"/>
+      <c r="R61" s="11" t="n"/>
+      <c r="S61" s="11" t="n"/>
+      <c r="T61" s="11" t="n"/>
+      <c r="U61" s="11" t="n"/>
+      <c r="V61" s="11" t="n"/>
+      <c r="W61" s="11" t="n"/>
+      <c r="X61" s="11" t="n"/>
+      <c r="Y61" s="11" t="n"/>
+      <c r="Z61" s="11" t="n"/>
+      <c r="AA61" s="11" t="n"/>
+      <c r="AB61" s="11" t="n"/>
+      <c r="AC61" s="11" t="n"/>
+      <c r="AD61" s="11" t="n"/>
+      <c r="AE61" s="11" t="n"/>
+      <c r="AF61" s="11" t="n"/>
+      <c r="AG61" s="11" t="n"/>
+      <c r="AH61" s="11" t="n"/>
+      <c r="AI61" s="11" t="n"/>
+      <c r="AJ61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -42862,6 +44813,35 @@
           <t>Partner Opus Genetics</t>
         </is>
       </c>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N62" s="10" t="n"/>
+      <c r="O62" s="10" t="n"/>
+      <c r="P62" s="10" t="n"/>
+      <c r="Q62" s="11" t="n"/>
+      <c r="R62" s="11" t="n"/>
+      <c r="S62" s="11" t="n"/>
+      <c r="T62" s="11" t="n"/>
+      <c r="U62" s="11" t="n"/>
+      <c r="V62" s="11" t="n"/>
+      <c r="W62" s="11" t="n"/>
+      <c r="X62" s="11" t="n"/>
+      <c r="Y62" s="11" t="n"/>
+      <c r="Z62" s="11" t="n"/>
+      <c r="AA62" s="11" t="n"/>
+      <c r="AB62" s="11" t="n"/>
+      <c r="AC62" s="11" t="n"/>
+      <c r="AD62" s="11" t="n"/>
+      <c r="AE62" s="11" t="n"/>
+      <c r="AF62" s="11" t="n"/>
+      <c r="AG62" s="11" t="n"/>
+      <c r="AH62" s="11" t="n"/>
+      <c r="AI62" s="11" t="n"/>
+      <c r="AJ62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -42915,6 +44895,35 @@
           <t>Regulatory uncertainty on accelerated approval</t>
         </is>
       </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>無明確日期: BLA</t>
+        </is>
+      </c>
+      <c r="M63" s="11" t="n"/>
+      <c r="N63" s="11" t="n"/>
+      <c r="O63" s="11" t="n"/>
+      <c r="P63" s="11" t="n"/>
+      <c r="Q63" s="11" t="n"/>
+      <c r="R63" s="11" t="n"/>
+      <c r="S63" s="11" t="n"/>
+      <c r="T63" s="11" t="n"/>
+      <c r="U63" s="11" t="n"/>
+      <c r="V63" s="11" t="n"/>
+      <c r="W63" s="11" t="n"/>
+      <c r="X63" s="11" t="n"/>
+      <c r="Y63" s="11" t="n"/>
+      <c r="Z63" s="11" t="n"/>
+      <c r="AA63" s="11" t="n"/>
+      <c r="AB63" s="11" t="n"/>
+      <c r="AC63" s="11" t="n"/>
+      <c r="AD63" s="11" t="n"/>
+      <c r="AE63" s="11" t="n"/>
+      <c r="AF63" s="11" t="n"/>
+      <c r="AG63" s="11" t="n"/>
+      <c r="AH63" s="11" t="n"/>
+      <c r="AI63" s="11" t="n"/>
+      <c r="AJ63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -42964,6 +44973,35 @@
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M64" s="11" t="n"/>
+      <c r="N64" s="11" t="n"/>
+      <c r="O64" s="11" t="n"/>
+      <c r="P64" s="11" t="n"/>
+      <c r="Q64" s="11" t="n"/>
+      <c r="R64" s="11" t="n"/>
+      <c r="S64" s="11" t="n"/>
+      <c r="T64" s="11" t="n"/>
+      <c r="U64" s="11" t="n"/>
+      <c r="V64" s="11" t="n"/>
+      <c r="W64" s="11" t="n"/>
+      <c r="X64" s="11" t="n"/>
+      <c r="Y64" s="11" t="n"/>
+      <c r="Z64" s="11" t="n"/>
+      <c r="AA64" s="11" t="n"/>
+      <c r="AB64" s="11" t="n"/>
+      <c r="AC64" s="11" t="n"/>
+      <c r="AD64" s="11" t="n"/>
+      <c r="AE64" s="11" t="n"/>
+      <c r="AF64" s="11" t="n"/>
+      <c r="AG64" s="11" t="n"/>
+      <c r="AH64" s="11" t="n"/>
+      <c r="AI64" s="11" t="n"/>
+      <c r="AJ64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -43013,6 +45051,35 @@
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N65" s="10" t="n"/>
+      <c r="O65" s="10" t="n"/>
+      <c r="P65" s="10" t="n"/>
+      <c r="Q65" s="11" t="n"/>
+      <c r="R65" s="11" t="n"/>
+      <c r="S65" s="11" t="n"/>
+      <c r="T65" s="11" t="n"/>
+      <c r="U65" s="11" t="n"/>
+      <c r="V65" s="11" t="n"/>
+      <c r="W65" s="11" t="n"/>
+      <c r="X65" s="11" t="n"/>
+      <c r="Y65" s="11" t="n"/>
+      <c r="Z65" s="11" t="n"/>
+      <c r="AA65" s="11" t="n"/>
+      <c r="AB65" s="11" t="n"/>
+      <c r="AC65" s="11" t="n"/>
+      <c r="AD65" s="11" t="n"/>
+      <c r="AE65" s="11" t="n"/>
+      <c r="AF65" s="11" t="n"/>
+      <c r="AG65" s="11" t="n"/>
+      <c r="AH65" s="11" t="n"/>
+      <c r="AI65" s="11" t="n"/>
+      <c r="AJ65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -43062,6 +45129,35 @@
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M66" s="11" t="n"/>
+      <c r="N66" s="11" t="n"/>
+      <c r="O66" s="11" t="n"/>
+      <c r="P66" s="11" t="n"/>
+      <c r="Q66" s="11" t="n"/>
+      <c r="R66" s="11" t="n"/>
+      <c r="S66" s="11" t="n"/>
+      <c r="T66" s="11" t="n"/>
+      <c r="U66" s="11" t="n"/>
+      <c r="V66" s="11" t="n"/>
+      <c r="W66" s="11" t="n"/>
+      <c r="X66" s="11" t="n"/>
+      <c r="Y66" s="11" t="n"/>
+      <c r="Z66" s="11" t="n"/>
+      <c r="AA66" s="11" t="n"/>
+      <c r="AB66" s="11" t="n"/>
+      <c r="AC66" s="11" t="n"/>
+      <c r="AD66" s="11" t="n"/>
+      <c r="AE66" s="11" t="n"/>
+      <c r="AF66" s="11" t="n"/>
+      <c r="AG66" s="11" t="n"/>
+      <c r="AH66" s="11" t="n"/>
+      <c r="AI66" s="11" t="n"/>
+      <c r="AJ66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -43111,6 +45207,35 @@
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="9" t="inlineStr">
+        <is>
+          <t>Ph3</t>
+        </is>
+      </c>
+      <c r="N67" s="10" t="n"/>
+      <c r="O67" s="10" t="n"/>
+      <c r="P67" s="10" t="n"/>
+      <c r="Q67" s="11" t="n"/>
+      <c r="R67" s="11" t="n"/>
+      <c r="S67" s="11" t="n"/>
+      <c r="T67" s="11" t="n"/>
+      <c r="U67" s="11" t="n"/>
+      <c r="V67" s="11" t="n"/>
+      <c r="W67" s="11" t="n"/>
+      <c r="X67" s="11" t="n"/>
+      <c r="Y67" s="11" t="n"/>
+      <c r="Z67" s="11" t="n"/>
+      <c r="AA67" s="11" t="n"/>
+      <c r="AB67" s="11" t="n"/>
+      <c r="AC67" s="11" t="n"/>
+      <c r="AD67" s="11" t="n"/>
+      <c r="AE67" s="11" t="n"/>
+      <c r="AF67" s="11" t="n"/>
+      <c r="AG67" s="11" t="n"/>
+      <c r="AH67" s="11" t="n"/>
+      <c r="AI67" s="11" t="n"/>
+      <c r="AJ67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -43160,6 +45285,35 @@
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="12" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N68" s="13" t="n"/>
+      <c r="O68" s="13" t="n"/>
+      <c r="P68" s="13" t="n"/>
+      <c r="Q68" s="11" t="n"/>
+      <c r="R68" s="11" t="n"/>
+      <c r="S68" s="11" t="n"/>
+      <c r="T68" s="11" t="n"/>
+      <c r="U68" s="11" t="n"/>
+      <c r="V68" s="11" t="n"/>
+      <c r="W68" s="11" t="n"/>
+      <c r="X68" s="11" t="n"/>
+      <c r="Y68" s="11" t="n"/>
+      <c r="Z68" s="11" t="n"/>
+      <c r="AA68" s="11" t="n"/>
+      <c r="AB68" s="11" t="n"/>
+      <c r="AC68" s="11" t="n"/>
+      <c r="AD68" s="11" t="n"/>
+      <c r="AE68" s="11" t="n"/>
+      <c r="AF68" s="11" t="n"/>
+      <c r="AG68" s="11" t="n"/>
+      <c r="AH68" s="11" t="n"/>
+      <c r="AI68" s="11" t="n"/>
+      <c r="AJ68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -43213,6 +45367,35 @@
           <t>Partnered w/ Nippon Shinyaku</t>
         </is>
       </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M69" s="11" t="n"/>
+      <c r="N69" s="11" t="n"/>
+      <c r="O69" s="11" t="n"/>
+      <c r="P69" s="11" t="n"/>
+      <c r="Q69" s="11" t="n"/>
+      <c r="R69" s="11" t="n"/>
+      <c r="S69" s="11" t="n"/>
+      <c r="T69" s="11" t="n"/>
+      <c r="U69" s="11" t="n"/>
+      <c r="V69" s="11" t="n"/>
+      <c r="W69" s="11" t="n"/>
+      <c r="X69" s="11" t="n"/>
+      <c r="Y69" s="11" t="n"/>
+      <c r="Z69" s="11" t="n"/>
+      <c r="AA69" s="11" t="n"/>
+      <c r="AB69" s="11" t="n"/>
+      <c r="AC69" s="11" t="n"/>
+      <c r="AD69" s="11" t="n"/>
+      <c r="AE69" s="11" t="n"/>
+      <c r="AF69" s="11" t="n"/>
+      <c r="AG69" s="11" t="n"/>
+      <c r="AH69" s="11" t="n"/>
+      <c r="AI69" s="11" t="n"/>
+      <c r="AJ69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -43262,6 +45445,35 @@
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N70" s="10" t="n"/>
+      <c r="O70" s="10" t="n"/>
+      <c r="P70" s="10" t="n"/>
+      <c r="Q70" s="11" t="n"/>
+      <c r="R70" s="11" t="n"/>
+      <c r="S70" s="11" t="n"/>
+      <c r="T70" s="11" t="n"/>
+      <c r="U70" s="11" t="n"/>
+      <c r="V70" s="11" t="n"/>
+      <c r="W70" s="11" t="n"/>
+      <c r="X70" s="11" t="n"/>
+      <c r="Y70" s="11" t="n"/>
+      <c r="Z70" s="11" t="n"/>
+      <c r="AA70" s="11" t="n"/>
+      <c r="AB70" s="11" t="n"/>
+      <c r="AC70" s="11" t="n"/>
+      <c r="AD70" s="11" t="n"/>
+      <c r="AE70" s="11" t="n"/>
+      <c r="AF70" s="11" t="n"/>
+      <c r="AG70" s="11" t="n"/>
+      <c r="AH70" s="11" t="n"/>
+      <c r="AI70" s="11" t="n"/>
+      <c r="AJ70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -43311,6 +45523,35 @@
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="12" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N71" s="13" t="n"/>
+      <c r="O71" s="13" t="n"/>
+      <c r="P71" s="13" t="n"/>
+      <c r="Q71" s="11" t="n"/>
+      <c r="R71" s="11" t="n"/>
+      <c r="S71" s="11" t="n"/>
+      <c r="T71" s="11" t="n"/>
+      <c r="U71" s="11" t="n"/>
+      <c r="V71" s="11" t="n"/>
+      <c r="W71" s="11" t="n"/>
+      <c r="X71" s="11" t="n"/>
+      <c r="Y71" s="11" t="n"/>
+      <c r="Z71" s="11" t="n"/>
+      <c r="AA71" s="11" t="n"/>
+      <c r="AB71" s="11" t="n"/>
+      <c r="AC71" s="11" t="n"/>
+      <c r="AD71" s="11" t="n"/>
+      <c r="AE71" s="11" t="n"/>
+      <c r="AF71" s="11" t="n"/>
+      <c r="AG71" s="11" t="n"/>
+      <c r="AH71" s="11" t="n"/>
+      <c r="AI71" s="11" t="n"/>
+      <c r="AJ71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -43360,6 +45601,35 @@
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N72" s="10" t="n"/>
+      <c r="O72" s="10" t="n"/>
+      <c r="P72" s="10" t="n"/>
+      <c r="Q72" s="11" t="n"/>
+      <c r="R72" s="11" t="n"/>
+      <c r="S72" s="11" t="n"/>
+      <c r="T72" s="11" t="n"/>
+      <c r="U72" s="11" t="n"/>
+      <c r="V72" s="11" t="n"/>
+      <c r="W72" s="11" t="n"/>
+      <c r="X72" s="11" t="n"/>
+      <c r="Y72" s="11" t="n"/>
+      <c r="Z72" s="11" t="n"/>
+      <c r="AA72" s="11" t="n"/>
+      <c r="AB72" s="11" t="n"/>
+      <c r="AC72" s="11" t="n"/>
+      <c r="AD72" s="11" t="n"/>
+      <c r="AE72" s="11" t="n"/>
+      <c r="AF72" s="11" t="n"/>
+      <c r="AG72" s="11" t="n"/>
+      <c r="AH72" s="11" t="n"/>
+      <c r="AI72" s="11" t="n"/>
+      <c r="AJ72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -43409,6 +45679,35 @@
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="14" t="inlineStr">
+        <is>
+          <t>逾期未發生: BLA</t>
+        </is>
+      </c>
+      <c r="M73" s="11" t="n"/>
+      <c r="N73" s="11" t="n"/>
+      <c r="O73" s="11" t="n"/>
+      <c r="P73" s="11" t="n"/>
+      <c r="Q73" s="11" t="n"/>
+      <c r="R73" s="11" t="n"/>
+      <c r="S73" s="11" t="n"/>
+      <c r="T73" s="11" t="n"/>
+      <c r="U73" s="11" t="n"/>
+      <c r="V73" s="11" t="n"/>
+      <c r="W73" s="11" t="n"/>
+      <c r="X73" s="11" t="n"/>
+      <c r="Y73" s="11" t="n"/>
+      <c r="Z73" s="11" t="n"/>
+      <c r="AA73" s="11" t="n"/>
+      <c r="AB73" s="11" t="n"/>
+      <c r="AC73" s="11" t="n"/>
+      <c r="AD73" s="11" t="n"/>
+      <c r="AE73" s="11" t="n"/>
+      <c r="AF73" s="11" t="n"/>
+      <c r="AG73" s="11" t="n"/>
+      <c r="AH73" s="11" t="n"/>
+      <c r="AI73" s="11" t="n"/>
+      <c r="AJ73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -43458,6 +45757,35 @@
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M74" s="11" t="n"/>
+      <c r="N74" s="11" t="n"/>
+      <c r="O74" s="11" t="n"/>
+      <c r="P74" s="11" t="n"/>
+      <c r="Q74" s="11" t="n"/>
+      <c r="R74" s="11" t="n"/>
+      <c r="S74" s="11" t="n"/>
+      <c r="T74" s="11" t="n"/>
+      <c r="U74" s="11" t="n"/>
+      <c r="V74" s="11" t="n"/>
+      <c r="W74" s="11" t="n"/>
+      <c r="X74" s="11" t="n"/>
+      <c r="Y74" s="11" t="n"/>
+      <c r="Z74" s="11" t="n"/>
+      <c r="AA74" s="11" t="n"/>
+      <c r="AB74" s="11" t="n"/>
+      <c r="AC74" s="11" t="n"/>
+      <c r="AD74" s="11" t="n"/>
+      <c r="AE74" s="11" t="n"/>
+      <c r="AF74" s="11" t="n"/>
+      <c r="AG74" s="11" t="n"/>
+      <c r="AH74" s="11" t="n"/>
+      <c r="AI74" s="11" t="n"/>
+      <c r="AJ74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -43511,6 +45839,35 @@
           <t>Single Ph3 in Bangladesh; RWE comparator risk</t>
         </is>
       </c>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N75" s="10" t="n"/>
+      <c r="O75" s="10" t="n"/>
+      <c r="P75" s="10" t="n"/>
+      <c r="Q75" s="11" t="n"/>
+      <c r="R75" s="11" t="n"/>
+      <c r="S75" s="11" t="n"/>
+      <c r="T75" s="11" t="n"/>
+      <c r="U75" s="11" t="n"/>
+      <c r="V75" s="11" t="n"/>
+      <c r="W75" s="11" t="n"/>
+      <c r="X75" s="11" t="n"/>
+      <c r="Y75" s="11" t="n"/>
+      <c r="Z75" s="11" t="n"/>
+      <c r="AA75" s="11" t="n"/>
+      <c r="AB75" s="11" t="n"/>
+      <c r="AC75" s="11" t="n"/>
+      <c r="AD75" s="11" t="n"/>
+      <c r="AE75" s="11" t="n"/>
+      <c r="AF75" s="11" t="n"/>
+      <c r="AG75" s="11" t="n"/>
+      <c r="AH75" s="11" t="n"/>
+      <c r="AI75" s="11" t="n"/>
+      <c r="AJ75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -43560,6 +45917,35 @@
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M76" s="11" t="n"/>
+      <c r="N76" s="11" t="n"/>
+      <c r="O76" s="11" t="n"/>
+      <c r="P76" s="11" t="n"/>
+      <c r="Q76" s="11" t="n"/>
+      <c r="R76" s="11" t="n"/>
+      <c r="S76" s="11" t="n"/>
+      <c r="T76" s="11" t="n"/>
+      <c r="U76" s="11" t="n"/>
+      <c r="V76" s="11" t="n"/>
+      <c r="W76" s="11" t="n"/>
+      <c r="X76" s="11" t="n"/>
+      <c r="Y76" s="11" t="n"/>
+      <c r="Z76" s="11" t="n"/>
+      <c r="AA76" s="11" t="n"/>
+      <c r="AB76" s="11" t="n"/>
+      <c r="AC76" s="11" t="n"/>
+      <c r="AD76" s="11" t="n"/>
+      <c r="AE76" s="11" t="n"/>
+      <c r="AF76" s="11" t="n"/>
+      <c r="AG76" s="11" t="n"/>
+      <c r="AH76" s="11" t="n"/>
+      <c r="AI76" s="11" t="n"/>
+      <c r="AJ76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -43609,6 +45995,35 @@
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="9" t="inlineStr">
+        <is>
+          <t>BLA</t>
+        </is>
+      </c>
+      <c r="N77" s="10" t="n"/>
+      <c r="O77" s="10" t="n"/>
+      <c r="P77" s="10" t="n"/>
+      <c r="Q77" s="11" t="n"/>
+      <c r="R77" s="11" t="n"/>
+      <c r="S77" s="11" t="n"/>
+      <c r="T77" s="11" t="n"/>
+      <c r="U77" s="11" t="n"/>
+      <c r="V77" s="11" t="n"/>
+      <c r="W77" s="11" t="n"/>
+      <c r="X77" s="11" t="n"/>
+      <c r="Y77" s="11" t="n"/>
+      <c r="Z77" s="11" t="n"/>
+      <c r="AA77" s="11" t="n"/>
+      <c r="AB77" s="11" t="n"/>
+      <c r="AC77" s="11" t="n"/>
+      <c r="AD77" s="11" t="n"/>
+      <c r="AE77" s="11" t="n"/>
+      <c r="AF77" s="11" t="n"/>
+      <c r="AG77" s="11" t="n"/>
+      <c r="AH77" s="11" t="n"/>
+      <c r="AI77" s="11" t="n"/>
+      <c r="AJ77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -43658,6 +46073,35 @@
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>決定</t>
+        </is>
+      </c>
+      <c r="N78" s="10" t="n"/>
+      <c r="O78" s="10" t="n"/>
+      <c r="P78" s="10" t="n"/>
+      <c r="Q78" s="11" t="n"/>
+      <c r="R78" s="11" t="n"/>
+      <c r="S78" s="11" t="n"/>
+      <c r="T78" s="11" t="n"/>
+      <c r="U78" s="11" t="n"/>
+      <c r="V78" s="11" t="n"/>
+      <c r="W78" s="11" t="n"/>
+      <c r="X78" s="11" t="n"/>
+      <c r="Y78" s="11" t="n"/>
+      <c r="Z78" s="11" t="n"/>
+      <c r="AA78" s="11" t="n"/>
+      <c r="AB78" s="11" t="n"/>
+      <c r="AC78" s="11" t="n"/>
+      <c r="AD78" s="11" t="n"/>
+      <c r="AE78" s="11" t="n"/>
+      <c r="AF78" s="11" t="n"/>
+      <c r="AG78" s="11" t="n"/>
+      <c r="AH78" s="11" t="n"/>
+      <c r="AI78" s="11" t="n"/>
+      <c r="AJ78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -43707,6 +46151,35 @@
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M79" s="11" t="n"/>
+      <c r="N79" s="11" t="n"/>
+      <c r="O79" s="11" t="n"/>
+      <c r="P79" s="11" t="n"/>
+      <c r="Q79" s="11" t="n"/>
+      <c r="R79" s="11" t="n"/>
+      <c r="S79" s="11" t="n"/>
+      <c r="T79" s="11" t="n"/>
+      <c r="U79" s="11" t="n"/>
+      <c r="V79" s="11" t="n"/>
+      <c r="W79" s="11" t="n"/>
+      <c r="X79" s="11" t="n"/>
+      <c r="Y79" s="11" t="n"/>
+      <c r="Z79" s="11" t="n"/>
+      <c r="AA79" s="11" t="n"/>
+      <c r="AB79" s="11" t="n"/>
+      <c r="AC79" s="11" t="n"/>
+      <c r="AD79" s="11" t="n"/>
+      <c r="AE79" s="11" t="n"/>
+      <c r="AF79" s="11" t="n"/>
+      <c r="AG79" s="11" t="n"/>
+      <c r="AH79" s="11" t="n"/>
+      <c r="AI79" s="11" t="n"/>
+      <c r="AJ79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -43760,6 +46233,35 @@
           <t>Illuccix approved 2022</t>
         </is>
       </c>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>重交</t>
+        </is>
+      </c>
+      <c r="N80" s="10" t="n"/>
+      <c r="O80" s="10" t="n"/>
+      <c r="P80" s="10" t="n"/>
+      <c r="Q80" s="11" t="n"/>
+      <c r="R80" s="11" t="n"/>
+      <c r="S80" s="11" t="n"/>
+      <c r="T80" s="11" t="n"/>
+      <c r="U80" s="11" t="n"/>
+      <c r="V80" s="11" t="n"/>
+      <c r="W80" s="11" t="n"/>
+      <c r="X80" s="11" t="n"/>
+      <c r="Y80" s="11" t="n"/>
+      <c r="Z80" s="11" t="n"/>
+      <c r="AA80" s="11" t="n"/>
+      <c r="AB80" s="11" t="n"/>
+      <c r="AC80" s="11" t="n"/>
+      <c r="AD80" s="11" t="n"/>
+      <c r="AE80" s="11" t="n"/>
+      <c r="AF80" s="11" t="n"/>
+      <c r="AG80" s="11" t="n"/>
+      <c r="AH80" s="11" t="n"/>
+      <c r="AI80" s="11" t="n"/>
+      <c r="AJ80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -43813,6 +46315,35 @@
           <t>Licensed from Abbisko</t>
         </is>
       </c>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="12" t="inlineStr">
+        <is>
+          <t>NDA</t>
+        </is>
+      </c>
+      <c r="N81" s="13" t="n"/>
+      <c r="O81" s="13" t="n"/>
+      <c r="P81" s="13" t="n"/>
+      <c r="Q81" s="11" t="n"/>
+      <c r="R81" s="11" t="n"/>
+      <c r="S81" s="11" t="n"/>
+      <c r="T81" s="11" t="n"/>
+      <c r="U81" s="11" t="n"/>
+      <c r="V81" s="11" t="n"/>
+      <c r="W81" s="11" t="n"/>
+      <c r="X81" s="11" t="n"/>
+      <c r="Y81" s="11" t="n"/>
+      <c r="Z81" s="11" t="n"/>
+      <c r="AA81" s="11" t="n"/>
+      <c r="AB81" s="11" t="n"/>
+      <c r="AC81" s="11" t="n"/>
+      <c r="AD81" s="11" t="n"/>
+      <c r="AE81" s="11" t="n"/>
+      <c r="AF81" s="11" t="n"/>
+      <c r="AG81" s="11" t="n"/>
+      <c r="AH81" s="11" t="n"/>
+      <c r="AI81" s="11" t="n"/>
+      <c r="AJ81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -43862,6 +46393,35 @@
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>CVOT</t>
+        </is>
+      </c>
+      <c r="N82" s="10" t="n"/>
+      <c r="O82" s="10" t="n"/>
+      <c r="P82" s="10" t="n"/>
+      <c r="Q82" s="11" t="n"/>
+      <c r="R82" s="11" t="n"/>
+      <c r="S82" s="11" t="n"/>
+      <c r="T82" s="11" t="n"/>
+      <c r="U82" s="11" t="n"/>
+      <c r="V82" s="11" t="n"/>
+      <c r="W82" s="11" t="n"/>
+      <c r="X82" s="11" t="n"/>
+      <c r="Y82" s="11" t="n"/>
+      <c r="Z82" s="11" t="n"/>
+      <c r="AA82" s="11" t="n"/>
+      <c r="AB82" s="11" t="n"/>
+      <c r="AC82" s="11" t="n"/>
+      <c r="AD82" s="11" t="n"/>
+      <c r="AE82" s="11" t="n"/>
+      <c r="AF82" s="11" t="n"/>
+      <c r="AG82" s="11" t="n"/>
+      <c r="AH82" s="11" t="n"/>
+      <c r="AI82" s="11" t="n"/>
+      <c r="AJ82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -43911,9 +46471,38 @@
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>無待發生項目</t>
+        </is>
+      </c>
+      <c r="M83" s="11" t="n"/>
+      <c r="N83" s="11" t="n"/>
+      <c r="O83" s="11" t="n"/>
+      <c r="P83" s="11" t="n"/>
+      <c r="Q83" s="11" t="n"/>
+      <c r="R83" s="11" t="n"/>
+      <c r="S83" s="11" t="n"/>
+      <c r="T83" s="11" t="n"/>
+      <c r="U83" s="11" t="n"/>
+      <c r="V83" s="11" t="n"/>
+      <c r="W83" s="11" t="n"/>
+      <c r="X83" s="11" t="n"/>
+      <c r="Y83" s="11" t="n"/>
+      <c r="Z83" s="11" t="n"/>
+      <c r="AA83" s="11" t="n"/>
+      <c r="AB83" s="11" t="n"/>
+      <c r="AC83" s="11" t="n"/>
+      <c r="AD83" s="11" t="n"/>
+      <c r="AE83" s="11" t="n"/>
+      <c r="AF83" s="11" t="n"/>
+      <c r="AG83" s="11" t="n"/>
+      <c r="AH83" s="11" t="n"/>
+      <c r="AI83" s="11" t="n"/>
+      <c r="AJ83" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83"/>
+  <autoFilter ref="A1:L83"/>
   <conditionalFormatting sqref="C2:C83">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -44020,7 +46609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -44028,250 +46617,334 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>FDA 藥物申請 Pipeline — 美國上巿 / ADR 可交易公司 (Curated snapshot)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr"/>
-      <c r="B2" s="8" t="n"/>
+      <c r="A2" s="17" t="inlineStr"/>
+      <c r="B2" s="17" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>資料截點 Data as-of</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>知識截點約 2026 年中 (mid-2026)。標註『verify』的項目 = 該 PDUFA/決定日期在截點附近或之後，請以 FDA / 公司公告核實最新狀態。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>覆蓋範圍 Coverage</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>本表為『重點策展』(curated) 而非窮盡式 (exhaustive) 名單。美國上巿/ADR 生物製藥公司逾 700 家，本表收錄約 178 家、338 個候選藥，聚焦：(a) NDA/BLA 審批中、(b) Phase 3、(c) 具巿場意義的 Phase 2 及 2024-25 新獲批藥。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>資料來源 Sources</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>公司新聞稿/10-K/年報、FDA 新聞稿及 Drugs@FDA、ClinicalTrials.gov、BIO/Informa/QLS《Clinical Development Success Rates》、賣方研究對 TAM/峯值銷售的共識估計。本環境無法即時連接 openFDA / ClinicalTrials.gov API (網絡政策封鎖)，故未能自動核對。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr"/>
-      <c r="B6" s="8" t="n"/>
+      <c r="A6" s="17" t="inlineStr"/>
+      <c r="B6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>FDA 階段定義 Stage definitions</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr"/>
+      <c r="B7" s="17" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Approved (recent)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>2024 年中至 2026 年中獲 FDA 批准 (含加速批准)，列出以便追蹤標籤擴充/確認性試驗。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>NDA/BLA under review</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>已向 FDA 提交 NDA/BLA 或 sNDA/sBLA，等待 PDUFA 決定。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>NDA/BLA under review (CRL history)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>曾收 Complete Response Letter (CRL) 或 Refuse-to-File，現重新提交。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Phase 3 (positive readout, filing pending)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Ph3 達主要終點，尚未提交。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Phase 3 / Phase 2/3 / Phase 2 / Phase 1/2</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>按 ClinicalTrials.gov 登記之最高階段。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr"/>
-      <c r="B13" s="8" t="n"/>
+      <c r="A13" s="17" t="inlineStr"/>
+      <c r="B13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>成功機會 PoS 方法 Probability-of-success method</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>基準率 Base rate (到最終獲批 LOA)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Approved (recent): 100%; NDA/BLA under review: 90%; NDA/BLA under review (CRL history): 75%; Phase 3 (positive readout, filing pending): 85%; Phase 3: 55%; Phase 2/3: 40%; Phase 2 (positive readout): 35%; Phase 2: 25%; Phase 1/2: 15%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>治療領域調整 TA adjustment (乘數)</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Oncology: x0.85; CNS/Psychiatry: x0.8; Neurology: x0.85; Cardiovascular: x0.95; Metabolic/Obesity: x1.0; Immunology: x1.0; Rare disease: x1.1; Hematology: x1.1; Infectious disease/Vaccine: x1.05; Ophthalmology: x0.95; Respiratory: x0.95; Nephrology: x0.95; Dermatology: x1.0; Gastroenterology: x0.95; Endocrinology: x1.0; Women's health: x1.0; Hepatology: x0.9</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>分析師覆寫 Analyst override</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>當有具體事件 (Ph3 失敗、CRL、安全事故、FDA 對數據集提出質疑) 時，以事件特定機率取代基準率，並於『PoS 依據』欄註明。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>PoS 上限</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>非已獲批項目上限 95%。</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr"/>
-      <c r="B19" s="8" t="n"/>
+      <c r="A19" s="17" t="inlineStr"/>
+      <c r="B19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>TAM 定義</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>以 US$ 十億計，代表該適應症/藥物類別之全球可及巿場 (峯值銷售或類別巿場規模)，多來自公司指引或賣方共識；同一公司內多個候選藥可能共享同一 TAM (例如肥胖 ~US$150bn)，故 Company Summary 內加總 TAM 為『未去重』僅供參考。</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr"/>
-      <c r="B21" s="8" t="n"/>
+      <c r="A21" s="17" t="inlineStr"/>
+      <c r="B21" s="17" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>催化劑切分 Catalyst split</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>『FDA Decisions Pending』分頁將催化劑按 2026-09-04 切為『已發生』與『待發生』兩欄。判斷準則：clause 陳述已完成動作 (positive / filed / accepted / CRL / RTF / approved / withdrawn / missed) 歸『已發生』；陳述預定動作 (decision / PDUFA / readout / filing) 而日期仍在未來則歸『待發生』；預定動作但日期或整個年度已過，亦歸『已發生』。</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>[日期已過，結果待核實]</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>該 PDUFA 日期已過，但落在本資料集知識截點 (約 2026 年中) 之後，故 FDA 的實際決定結果本表無從得知，必須自行核實。</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>24個月排程格 24-month schedule grid</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>『FDA Decisions Pending』分頁最右方為由 2026-09 至 2028-08 的月度格，每格一個月，把『待發生』欄的時間點填上。顏色深淺代表時間精度，並非重要性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  深藍 (月精度)</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>原文有明確年月或日期，例如 PDUFA Sep 18 2026 -&gt; 只填該月。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  中藍 (半年/季精度)</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>原文為 early / mid / late / H1 / H2 / Q1-Q4 + 年份，填該區間所有月份。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  淺藍 (年精度)</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>原文只有年份，例如 decision 2026 -&gt; 填該年全部月份 (2026 年由 9 月起計)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  最淺藍 (跨年區間)</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>原文為 2026-27 之類跨年區間，填整個區間。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  格內標籤</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>PDUFA / 決定 / 遞交 / NDA / BLA / 重交 / 數據 / CVOT / Ph3 / 批核，只標在區間第一格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>排程狀態欄 Schedule status</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>『無待發生項目』= 該藥的待發生欄為空 (通常因 PDUFA 日期已過而結果未知)；『逾期未發生』= 原文時窗完全早於 2026-09，該預定事件理應已發生卻無更新，需優先核實；『無明確日期』= 原文無可解析日期 (例如 path uncertain)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>免責聲明 Disclaimer</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>僅供研究參考，不構成投資建議。生物科技股價對 FDA 決定高度敏感，請以最新公告核實。</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>TradingView 連結 TradingView links</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>所有『代號 Ticker』欄位均已加上超連結，格式為 https://www.tradingview.com/chart/Q1c5VWwD/?symbol=&lt;ticker(小寫)&gt;，例如 ticker = NE -&gt; https://www.tradingview.com/chart/Q1c5VWwD/?symbol=ne 。ADR/OTC 代號在 TradingView 上可能需要加交易所前綴 (例如 OTC:RHHBY) 方能正確開圖，若連結未能載入請於 TradingView 內手動搜尋該代號。</t>
         </is>

</xml_diff>